<commit_message>
feat: Add QQOQCP synthesis for 2026 industrial organization missions in Markdown and HTML.
</commit_message>
<xml_diff>
--- a/OI/CV Bourges/PLANNING 2025 2026 PRF Décembre MODIFIE TRE RAN OK POUR NL Bourges.xlsx
+++ b/OI/CV Bourges/PLANNING 2025 2026 PRF Décembre MODIFIE TRE RAN OK POUR NL Bourges.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_hubert_poleformation-uimmcvdl_fr/Documents/Bureau/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/CV Bourges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="8_{65CE5636-56B4-491F-B8F0-4DF62A4688D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60CF26A3-7B92-4C03-B4FB-B3D9C0863B99}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{65CE5636-56B4-491F-B8F0-4DF62A4688D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8BD0433-F281-4329-AED4-1E85A79E6379}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{57C63110-A53C-4A27-AFD1-0C77926CCA02}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{57C63110-A53C-4A27-AFD1-0C77926CCA02}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -328,7 +328,7 @@
     <numFmt numFmtId="164" formatCode="[$-40C]mmmmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ d"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -496,6 +496,14 @@
       <color rgb="FFEE0000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="22">
@@ -846,7 +854,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1108,53 +1116,8 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1199,9 +1162,55 @@
     <xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1275,10 +1284,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1582,106 +1587,107 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AV68"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.46484375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" customWidth="1"/>
-    <col min="3" max="3" width="6.46484375" customWidth="1"/>
-    <col min="4" max="4" width="7.86328125" customWidth="1"/>
-    <col min="5" max="5" width="2.6640625" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" customWidth="1"/>
-    <col min="7" max="7" width="6.46484375" customWidth="1"/>
-    <col min="8" max="8" width="9.86328125" customWidth="1"/>
-    <col min="9" max="9" width="2.6640625" customWidth="1"/>
-    <col min="10" max="10" width="7.33203125" customWidth="1"/>
-    <col min="11" max="12" width="6.46484375" customWidth="1"/>
-    <col min="13" max="13" width="3.6640625" customWidth="1"/>
-    <col min="14" max="14" width="7.33203125" customWidth="1"/>
-    <col min="15" max="16" width="6.46484375" customWidth="1"/>
-    <col min="17" max="17" width="2.6640625" customWidth="1"/>
-    <col min="18" max="18" width="7.33203125" customWidth="1"/>
-    <col min="19" max="20" width="6.46484375" customWidth="1"/>
-    <col min="21" max="21" width="2.6640625" customWidth="1"/>
-    <col min="22" max="22" width="7.33203125" customWidth="1"/>
-    <col min="23" max="24" width="6.46484375" customWidth="1"/>
-    <col min="25" max="25" width="2.6640625" customWidth="1"/>
-    <col min="26" max="26" width="7.33203125" customWidth="1"/>
-    <col min="27" max="27" width="6.46484375" customWidth="1"/>
-    <col min="28" max="28" width="6.19921875" customWidth="1"/>
-    <col min="29" max="29" width="2.6640625" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="7.46484375" hidden="1" customWidth="1"/>
-    <col min="31" max="32" width="6.46484375" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="2.6640625" hidden="1" customWidth="1"/>
-    <col min="34" max="34" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="35" max="36" width="6.46484375" hidden="1" customWidth="1"/>
-    <col min="37" max="37" width="0.1328125" customWidth="1"/>
-    <col min="38" max="38" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="39" max="40" width="6.46484375" hidden="1" customWidth="1"/>
-    <col min="41" max="41" width="3.33203125" hidden="1" customWidth="1"/>
-    <col min="42" max="42" width="6.86328125" hidden="1" customWidth="1"/>
-    <col min="43" max="44" width="6.1328125" hidden="1" customWidth="1"/>
-    <col min="45" max="45" width="3.86328125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" customWidth="1"/>
+    <col min="3" max="3" width="6.42578125" customWidth="1"/>
+    <col min="4" max="4" width="7.85546875" customWidth="1"/>
+    <col min="5" max="5" width="2.7109375" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" customWidth="1"/>
+    <col min="7" max="7" width="6.42578125" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" customWidth="1"/>
+    <col min="9" max="9" width="2.7109375" customWidth="1"/>
+    <col min="10" max="10" width="7.28515625" customWidth="1"/>
+    <col min="11" max="12" width="6.42578125" customWidth="1"/>
+    <col min="13" max="13" width="3.7109375" customWidth="1"/>
+    <col min="14" max="14" width="7.28515625" customWidth="1"/>
+    <col min="15" max="16" width="6.42578125" customWidth="1"/>
+    <col min="17" max="17" width="2.7109375" customWidth="1"/>
+    <col min="18" max="18" width="7.28515625" customWidth="1"/>
+    <col min="19" max="19" width="6.42578125" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" customWidth="1"/>
+    <col min="21" max="21" width="2.7109375" customWidth="1"/>
+    <col min="22" max="22" width="7.28515625" customWidth="1"/>
+    <col min="23" max="24" width="6.42578125" customWidth="1"/>
+    <col min="25" max="25" width="2.7109375" customWidth="1"/>
+    <col min="26" max="26" width="7.28515625" customWidth="1"/>
+    <col min="27" max="27" width="6.42578125" customWidth="1"/>
+    <col min="28" max="28" width="6.140625" customWidth="1"/>
+    <col min="29" max="29" width="2.7109375" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="7.42578125" hidden="1" customWidth="1"/>
+    <col min="31" max="32" width="6.42578125" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="2.7109375" hidden="1" customWidth="1"/>
+    <col min="34" max="34" width="7.28515625" hidden="1" customWidth="1"/>
+    <col min="35" max="36" width="6.42578125" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="0.140625" customWidth="1"/>
+    <col min="38" max="38" width="7.28515625" hidden="1" customWidth="1"/>
+    <col min="39" max="40" width="6.42578125" hidden="1" customWidth="1"/>
+    <col min="41" max="41" width="3.28515625" hidden="1" customWidth="1"/>
+    <col min="42" max="42" width="6.85546875" hidden="1" customWidth="1"/>
+    <col min="43" max="44" width="6.140625" hidden="1" customWidth="1"/>
+    <col min="45" max="45" width="3.85546875" hidden="1" customWidth="1"/>
     <col min="46" max="46" width="7" hidden="1" customWidth="1"/>
-    <col min="47" max="47" width="9.1328125" hidden="1" customWidth="1"/>
-    <col min="48" max="48" width="6.19921875" hidden="1" customWidth="1"/>
+    <col min="47" max="47" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="48" max="48" width="6.140625" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" ht="20.65" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:48" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="98"/>
-      <c r="I1" s="98"/>
-      <c r="J1" s="98"/>
-      <c r="K1" s="98"/>
-      <c r="L1" s="98"/>
-      <c r="M1" s="98"/>
-      <c r="N1" s="98"/>
-      <c r="O1" s="98"/>
-      <c r="P1" s="98"/>
-      <c r="Q1" s="98"/>
-      <c r="R1" s="98"/>
-      <c r="S1" s="98"/>
-      <c r="T1" s="98"/>
-      <c r="U1" s="98"/>
-      <c r="V1" s="98"/>
-      <c r="W1" s="98"/>
-      <c r="X1" s="98"/>
-      <c r="Y1" s="98"/>
-      <c r="Z1" s="98"/>
-      <c r="AA1" s="98"/>
-      <c r="AB1" s="98"/>
-      <c r="AC1" s="98"/>
-      <c r="AD1" s="98"/>
-      <c r="AE1" s="98"/>
-      <c r="AF1" s="98"/>
-      <c r="AG1" s="98"/>
-      <c r="AH1" s="98"/>
-      <c r="AI1" s="98"/>
-      <c r="AJ1" s="98"/>
-      <c r="AK1" s="98"/>
-      <c r="AL1" s="98"/>
-      <c r="AM1" s="98"/>
-      <c r="AN1" s="98"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
+      <c r="H1" s="116"/>
+      <c r="I1" s="116"/>
+      <c r="J1" s="116"/>
+      <c r="K1" s="116"/>
+      <c r="L1" s="116"/>
+      <c r="M1" s="116"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="116"/>
+      <c r="P1" s="116"/>
+      <c r="Q1" s="116"/>
+      <c r="R1" s="116"/>
+      <c r="S1" s="116"/>
+      <c r="T1" s="116"/>
+      <c r="U1" s="116"/>
+      <c r="V1" s="116"/>
+      <c r="W1" s="116"/>
+      <c r="X1" s="116"/>
+      <c r="Y1" s="116"/>
+      <c r="Z1" s="116"/>
+      <c r="AA1" s="116"/>
+      <c r="AB1" s="116"/>
+      <c r="AC1" s="116"/>
+      <c r="AD1" s="116"/>
+      <c r="AE1" s="116"/>
+      <c r="AF1" s="116"/>
+      <c r="AG1" s="116"/>
+      <c r="AH1" s="116"/>
+      <c r="AI1" s="116"/>
+      <c r="AJ1" s="116"/>
+      <c r="AK1" s="116"/>
+      <c r="AL1" s="116"/>
+      <c r="AM1" s="116"/>
+      <c r="AN1" s="116"/>
       <c r="AO1" s="1"/>
       <c r="AP1" s="1"/>
       <c r="AQ1" s="1"/>
       <c r="AR1" s="1"/>
     </row>
-    <row r="2" spans="1:48" ht="17.25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="99"/>
-      <c r="I2" s="99"/>
-      <c r="J2" s="99"/>
+      <c r="H2" s="117"/>
+      <c r="I2" s="117"/>
+      <c r="J2" s="117"/>
       <c r="K2" s="1"/>
       <c r="L2" s="2" t="s">
         <v>0</v>
@@ -1719,7 +1725,7 @@
       <c r="AQ2" s="1"/>
       <c r="AR2" s="1"/>
     </row>
-    <row r="3" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="3"/>
       <c r="C3" s="1"/>
@@ -1727,9 +1733,9 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="99"/>
-      <c r="I3" s="99"/>
-      <c r="J3" s="99"/>
+      <c r="H3" s="117"/>
+      <c r="I3" s="117"/>
+      <c r="J3" s="117"/>
       <c r="K3" s="4" t="s">
         <v>1</v>
       </c>
@@ -1742,19 +1748,19 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="1"/>
-      <c r="S3" s="100"/>
-      <c r="T3" s="101"/>
-      <c r="U3" s="101"/>
-      <c r="V3" s="101"/>
-      <c r="W3" s="101"/>
-      <c r="X3" s="101"/>
-      <c r="Y3" s="101"/>
-      <c r="Z3" s="101"/>
-      <c r="AA3" s="101"/>
-      <c r="AB3" s="101"/>
-      <c r="AC3" s="101"/>
-      <c r="AD3" s="101"/>
-      <c r="AE3" s="101"/>
+      <c r="S3" s="118"/>
+      <c r="T3" s="119"/>
+      <c r="U3" s="119"/>
+      <c r="V3" s="119"/>
+      <c r="W3" s="119"/>
+      <c r="X3" s="119"/>
+      <c r="Y3" s="119"/>
+      <c r="Z3" s="119"/>
+      <c r="AA3" s="119"/>
+      <c r="AB3" s="119"/>
+      <c r="AC3" s="119"/>
+      <c r="AD3" s="119"/>
+      <c r="AE3" s="119"/>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
       <c r="AH3" s="1"/>
@@ -1769,7 +1775,7 @@
       <c r="AQ3" s="1"/>
       <c r="AR3" s="1"/>
     </row>
-    <row r="4" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="3"/>
       <c r="C4" s="1"/>
@@ -1819,7 +1825,7 @@
       <c r="AQ4" s="1"/>
       <c r="AR4" s="1"/>
     </row>
-    <row r="5" spans="1:48" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:48" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="6"/>
       <c r="C5" s="7"/>
@@ -1869,7 +1875,7 @@
       <c r="AQ5" s="1"/>
       <c r="AR5" s="1"/>
     </row>
-    <row r="6" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="3"/>
       <c r="C6" s="1"/>
@@ -1915,19 +1921,19 @@
       <c r="AQ6" s="1"/>
       <c r="AR6" s="1"/>
     </row>
-    <row r="7" spans="1:48" ht="18" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:48" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
-      <c r="B7" s="95" t="s">
+      <c r="B7" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="95"/>
-      <c r="D7" s="95"/>
-      <c r="E7" s="95"/>
-      <c r="F7" s="95"/>
-      <c r="G7" s="95"/>
-      <c r="H7" s="95"/>
-      <c r="I7" s="95"/>
-      <c r="J7" s="95"/>
+      <c r="C7" s="120"/>
+      <c r="D7" s="120"/>
+      <c r="E7" s="120"/>
+      <c r="F7" s="120"/>
+      <c r="G7" s="120"/>
+      <c r="H7" s="120"/>
+      <c r="I7" s="120"/>
+      <c r="J7" s="120"/>
       <c r="K7" s="9">
         <f>C45+G45+K45+O45+S45+W45+AA45+AM45+AQ45+AU45</f>
         <v>595</v>
@@ -1970,19 +1976,19 @@
       <c r="AQ7" s="1"/>
       <c r="AR7" s="1"/>
     </row>
-    <row r="8" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="95" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="95"/>
-      <c r="D8" s="95"/>
-      <c r="E8" s="95"/>
-      <c r="F8" s="95"/>
-      <c r="G8" s="95"/>
-      <c r="H8" s="95"/>
-      <c r="I8" s="95"/>
-      <c r="J8" s="95"/>
+      <c r="B8" s="120" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="120"/>
+      <c r="D8" s="120"/>
+      <c r="E8" s="120"/>
+      <c r="F8" s="120"/>
+      <c r="G8" s="120"/>
+      <c r="H8" s="120"/>
+      <c r="I8" s="120"/>
+      <c r="J8" s="120"/>
       <c r="K8" s="5">
         <f>D45+H45+L45+P45+T45+X45+AB45+AN45</f>
         <v>259</v>
@@ -1995,17 +2001,17 @@
       </c>
       <c r="N8" s="4"/>
       <c r="O8" s="5"/>
-      <c r="P8" s="102"/>
-      <c r="Q8" s="102"/>
-      <c r="R8" s="102"/>
-      <c r="S8" s="102"/>
+      <c r="P8" s="121"/>
+      <c r="Q8" s="121"/>
+      <c r="R8" s="121"/>
+      <c r="S8" s="121"/>
       <c r="T8" s="10"/>
       <c r="U8" s="10"/>
       <c r="V8" s="10"/>
-      <c r="W8" s="102"/>
-      <c r="X8" s="102"/>
-      <c r="Y8" s="102"/>
-      <c r="Z8" s="102"/>
+      <c r="W8" s="121"/>
+      <c r="X8" s="121"/>
+      <c r="Y8" s="121"/>
+      <c r="Z8" s="121"/>
       <c r="AA8" s="10"/>
       <c r="AB8" s="10"/>
       <c r="AC8" s="10"/>
@@ -2025,19 +2031,19 @@
       <c r="AQ8" s="1"/>
       <c r="AR8" s="1"/>
     </row>
-    <row r="9" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="95" t="s">
+      <c r="B9" s="120" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="95"/>
-      <c r="D9" s="95"/>
-      <c r="E9" s="95"/>
-      <c r="F9" s="95"/>
-      <c r="G9" s="95"/>
-      <c r="H9" s="95"/>
-      <c r="I9" s="95"/>
-      <c r="J9" s="95"/>
+      <c r="C9" s="120"/>
+      <c r="D9" s="120"/>
+      <c r="E9" s="120"/>
+      <c r="F9" s="120"/>
+      <c r="G9" s="120"/>
+      <c r="H9" s="120"/>
+      <c r="I9" s="120"/>
+      <c r="J9" s="120"/>
       <c r="K9" s="5">
         <f>K7+K8</f>
         <v>854</v>
@@ -2080,7 +2086,7 @@
       <c r="AQ9" s="1"/>
       <c r="AR9" s="1"/>
     </row>
-    <row r="10" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="3"/>
       <c r="C10" s="1"/>
@@ -2126,171 +2132,171 @@
       <c r="AQ10" s="1"/>
       <c r="AR10" s="1"/>
     </row>
-    <row r="11" spans="1:48" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="103" t="s">
+    <row r="11" spans="1:48" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="104"/>
-      <c r="C11" s="104"/>
-      <c r="D11" s="105"/>
-      <c r="E11" s="103" t="s">
+      <c r="B11" s="110"/>
+      <c r="C11" s="110"/>
+      <c r="D11" s="111"/>
+      <c r="E11" s="109" t="s">
         <v>58</v>
       </c>
-      <c r="F11" s="104"/>
-      <c r="G11" s="104"/>
-      <c r="H11" s="105"/>
-      <c r="I11" s="103" t="s">
+      <c r="F11" s="110"/>
+      <c r="G11" s="110"/>
+      <c r="H11" s="111"/>
+      <c r="I11" s="109" t="s">
         <v>59</v>
       </c>
-      <c r="J11" s="104"/>
-      <c r="K11" s="104"/>
-      <c r="L11" s="105"/>
-      <c r="M11" s="103" t="s">
+      <c r="J11" s="110"/>
+      <c r="K11" s="110"/>
+      <c r="L11" s="111"/>
+      <c r="M11" s="109" t="s">
         <v>60</v>
       </c>
-      <c r="N11" s="104"/>
-      <c r="O11" s="104"/>
-      <c r="P11" s="105"/>
-      <c r="Q11" s="103" t="s">
+      <c r="N11" s="110"/>
+      <c r="O11" s="110"/>
+      <c r="P11" s="111"/>
+      <c r="Q11" s="109" t="s">
         <v>61</v>
       </c>
-      <c r="R11" s="104"/>
-      <c r="S11" s="104"/>
-      <c r="T11" s="105"/>
-      <c r="U11" s="103" t="s">
+      <c r="R11" s="110"/>
+      <c r="S11" s="110"/>
+      <c r="T11" s="111"/>
+      <c r="U11" s="109" t="s">
         <v>62</v>
       </c>
-      <c r="V11" s="104"/>
-      <c r="W11" s="104"/>
-      <c r="X11" s="105"/>
-      <c r="Y11" s="103" t="s">
+      <c r="V11" s="110"/>
+      <c r="W11" s="110"/>
+      <c r="X11" s="111"/>
+      <c r="Y11" s="109" t="s">
         <v>75</v>
       </c>
-      <c r="Z11" s="104"/>
-      <c r="AA11" s="104"/>
-      <c r="AB11" s="105"/>
-      <c r="AC11" s="103" t="s">
+      <c r="Z11" s="110"/>
+      <c r="AA11" s="110"/>
+      <c r="AB11" s="111"/>
+      <c r="AC11" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="AD11" s="104"/>
-      <c r="AE11" s="104"/>
-      <c r="AF11" s="105"/>
-      <c r="AG11" s="103" t="s">
+      <c r="AD11" s="110"/>
+      <c r="AE11" s="110"/>
+      <c r="AF11" s="111"/>
+      <c r="AG11" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="AH11" s="104"/>
-      <c r="AI11" s="104"/>
-      <c r="AJ11" s="105"/>
-      <c r="AK11" s="103" t="s">
+      <c r="AH11" s="110"/>
+      <c r="AI11" s="110"/>
+      <c r="AJ11" s="111"/>
+      <c r="AK11" s="109" t="s">
         <v>61</v>
       </c>
-      <c r="AL11" s="104"/>
-      <c r="AM11" s="104"/>
-      <c r="AN11" s="105"/>
-      <c r="AO11" s="103" t="s">
+      <c r="AL11" s="110"/>
+      <c r="AM11" s="110"/>
+      <c r="AN11" s="111"/>
+      <c r="AO11" s="109" t="s">
         <v>62</v>
       </c>
-      <c r="AP11" s="104"/>
-      <c r="AQ11" s="104"/>
-      <c r="AR11" s="105"/>
-      <c r="AS11" s="103" t="s">
+      <c r="AP11" s="110"/>
+      <c r="AQ11" s="110"/>
+      <c r="AR11" s="111"/>
+      <c r="AS11" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="AT11" s="104"/>
-      <c r="AU11" s="104"/>
-      <c r="AV11" s="105"/>
+      <c r="AT11" s="110"/>
+      <c r="AU11" s="110"/>
+      <c r="AV11" s="111"/>
     </row>
-    <row r="12" spans="1:48" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="96"/>
-      <c r="B12" s="97"/>
+    <row r="12" spans="1:48" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="112"/>
+      <c r="B12" s="108"/>
       <c r="C12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="96"/>
-      <c r="F12" s="97"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="108"/>
       <c r="G12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="H12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="96"/>
-      <c r="J12" s="97"/>
+      <c r="I12" s="112"/>
+      <c r="J12" s="108"/>
       <c r="K12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="L12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="M12" s="96"/>
-      <c r="N12" s="97"/>
+      <c r="M12" s="112"/>
+      <c r="N12" s="108"/>
       <c r="O12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="P12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="Q12" s="96"/>
-      <c r="R12" s="97"/>
+      <c r="Q12" s="112"/>
+      <c r="R12" s="108"/>
       <c r="S12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="T12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="U12" s="96"/>
-      <c r="V12" s="97"/>
+      <c r="U12" s="112"/>
+      <c r="V12" s="108"/>
       <c r="W12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="X12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="Y12" s="96"/>
-      <c r="Z12" s="97"/>
+      <c r="Y12" s="112"/>
+      <c r="Z12" s="108"/>
       <c r="AA12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="AB12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="AC12" s="96"/>
-      <c r="AD12" s="97"/>
+      <c r="AC12" s="112"/>
+      <c r="AD12" s="108"/>
       <c r="AE12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="AF12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="AG12" s="96"/>
-      <c r="AH12" s="97"/>
+      <c r="AG12" s="112"/>
+      <c r="AH12" s="108"/>
       <c r="AI12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="AJ12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="AK12" s="96"/>
-      <c r="AL12" s="97"/>
+      <c r="AK12" s="112"/>
+      <c r="AL12" s="108"/>
       <c r="AM12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="AN12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="AO12" s="106"/>
-      <c r="AP12" s="97"/>
+      <c r="AO12" s="107"/>
+      <c r="AP12" s="108"/>
       <c r="AQ12" s="12" t="s">
         <v>11</v>
       </c>
       <c r="AR12" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="AS12" s="106"/>
-      <c r="AT12" s="97"/>
+      <c r="AS12" s="107"/>
+      <c r="AT12" s="108"/>
       <c r="AU12" s="12" t="s">
         <v>11</v>
       </c>
@@ -2298,8 +2304,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="93" t="s">
+    <row r="13" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="113" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="16">
@@ -2311,7 +2317,7 @@
       <c r="D13" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E13" s="93" t="s">
+      <c r="E13" s="113" t="s">
         <v>64</v>
       </c>
       <c r="F13" s="14">
@@ -2331,7 +2337,7 @@
       </c>
       <c r="O13" s="21"/>
       <c r="P13" s="59"/>
-      <c r="Q13" s="94" t="s">
+      <c r="Q13" s="122" t="s">
         <v>13</v>
       </c>
       <c r="R13" s="16">
@@ -2341,7 +2347,7 @@
       <c r="T13" s="24">
         <v>7</v>
       </c>
-      <c r="U13" s="93" t="s">
+      <c r="U13" s="113" t="s">
         <v>14</v>
       </c>
       <c r="V13" s="14">
@@ -2349,7 +2355,7 @@
       </c>
       <c r="W13" s="21"/>
       <c r="X13" s="20"/>
-      <c r="Y13" s="93" t="s">
+      <c r="Y13" s="113" t="s">
         <v>76</v>
       </c>
       <c r="Z13" s="16">
@@ -2357,7 +2363,7 @@
       </c>
       <c r="AA13" s="23"/>
       <c r="AB13" s="19"/>
-      <c r="AC13" s="94" t="s">
+      <c r="AC13" s="122" t="s">
         <v>15</v>
       </c>
       <c r="AD13" s="16">
@@ -2365,7 +2371,7 @@
       </c>
       <c r="AE13" s="23"/>
       <c r="AF13" s="27"/>
-      <c r="AG13" s="94" t="s">
+      <c r="AG13" s="122" t="s">
         <v>16</v>
       </c>
       <c r="AH13" s="16">
@@ -2373,7 +2379,7 @@
       </c>
       <c r="AI13" s="60"/>
       <c r="AJ13" s="32"/>
-      <c r="AK13" s="94" t="s">
+      <c r="AK13" s="122" t="s">
         <v>13</v>
       </c>
       <c r="AL13" s="16">
@@ -2381,13 +2387,13 @@
       </c>
       <c r="AM13" s="23"/>
       <c r="AN13" s="19"/>
-      <c r="AO13" s="93"/>
+      <c r="AO13" s="113"/>
       <c r="AP13" s="14">
         <v>46143</v>
       </c>
       <c r="AQ13" s="25"/>
       <c r="AR13" s="26"/>
-      <c r="AS13" s="94" t="s">
+      <c r="AS13" s="122" t="s">
         <v>17</v>
       </c>
       <c r="AT13" s="16">
@@ -2396,8 +2402,8 @@
       <c r="AU13" s="21"/>
       <c r="AV13" s="15"/>
     </row>
-    <row r="14" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="91"/>
+    <row r="14" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="114"/>
       <c r="B14" s="16">
         <v>45902</v>
       </c>
@@ -2407,13 +2413,13 @@
       <c r="D14" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="91"/>
+      <c r="E14" s="114"/>
       <c r="F14" s="72">
         <v>46024</v>
       </c>
       <c r="G14" s="83"/>
       <c r="H14" s="85"/>
-      <c r="I14" s="93" t="s">
+      <c r="I14" s="113" t="s">
         <v>69</v>
       </c>
       <c r="J14" s="16">
@@ -2425,7 +2431,7 @@
       <c r="L14" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M14" s="93" t="s">
+      <c r="M14" s="113" t="s">
         <v>18</v>
       </c>
       <c r="N14" s="16">
@@ -2435,7 +2441,7 @@
       <c r="P14" s="24">
         <v>7</v>
       </c>
-      <c r="Q14" s="94"/>
+      <c r="Q14" s="122"/>
       <c r="R14" s="16">
         <v>45932</v>
       </c>
@@ -2443,51 +2449,51 @@
       <c r="T14" s="24">
         <v>7</v>
       </c>
-      <c r="U14" s="91"/>
+      <c r="U14" s="114"/>
       <c r="V14" s="14">
         <v>45871</v>
       </c>
       <c r="W14" s="21"/>
       <c r="X14" s="22"/>
-      <c r="Y14" s="91"/>
+      <c r="Y14" s="114"/>
       <c r="Z14" s="16">
         <v>45902</v>
       </c>
       <c r="AA14" s="23"/>
       <c r="AB14" s="19"/>
-      <c r="AC14" s="94"/>
+      <c r="AC14" s="122"/>
       <c r="AD14" s="16">
         <v>45932</v>
       </c>
       <c r="AE14" s="23"/>
       <c r="AF14" s="27"/>
-      <c r="AG14" s="94"/>
+      <c r="AG14" s="122"/>
       <c r="AH14" s="16">
         <v>45902</v>
       </c>
       <c r="AI14" s="23"/>
       <c r="AJ14" s="18"/>
-      <c r="AK14" s="94"/>
+      <c r="AK14" s="122"/>
       <c r="AL14" s="16">
         <v>46114</v>
       </c>
       <c r="AM14" s="23"/>
       <c r="AN14" s="19"/>
-      <c r="AO14" s="91"/>
+      <c r="AO14" s="114"/>
       <c r="AP14" s="14">
         <v>46144</v>
       </c>
       <c r="AQ14" s="21"/>
       <c r="AR14" s="22"/>
-      <c r="AS14" s="94"/>
+      <c r="AS14" s="122"/>
       <c r="AT14" s="16">
         <v>45993</v>
       </c>
       <c r="AU14" s="23"/>
       <c r="AV14" s="29"/>
     </row>
-    <row r="15" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="91"/>
+    <row r="15" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="114"/>
       <c r="B15" s="16">
         <v>45903</v>
       </c>
@@ -2497,13 +2503,13 @@
       <c r="D15" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="91"/>
+      <c r="E15" s="114"/>
       <c r="F15" s="14">
         <v>46025</v>
       </c>
       <c r="G15" s="21"/>
       <c r="H15" s="59"/>
-      <c r="I15" s="91"/>
+      <c r="I15" s="114"/>
       <c r="J15" s="16">
         <v>46056</v>
       </c>
@@ -2513,7 +2519,7 @@
       <c r="L15" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M15" s="91"/>
+      <c r="M15" s="114"/>
       <c r="N15" s="16">
         <v>46084</v>
       </c>
@@ -2521,7 +2527,7 @@
       <c r="P15" s="24">
         <v>7</v>
       </c>
-      <c r="Q15" s="94"/>
+      <c r="Q15" s="122"/>
       <c r="R15" s="16">
         <v>45933</v>
       </c>
@@ -2529,51 +2535,51 @@
       <c r="T15" s="24">
         <v>7</v>
       </c>
-      <c r="U15" s="92"/>
+      <c r="U15" s="115"/>
       <c r="V15" s="14">
         <v>45872</v>
       </c>
       <c r="W15" s="15"/>
       <c r="X15" s="20"/>
-      <c r="Y15" s="91"/>
+      <c r="Y15" s="114"/>
       <c r="Z15" s="16">
         <v>45903</v>
       </c>
       <c r="AA15" s="23"/>
       <c r="AB15" s="19"/>
-      <c r="AC15" s="94"/>
+      <c r="AC15" s="122"/>
       <c r="AD15" s="16">
         <v>45933</v>
       </c>
       <c r="AE15" s="23"/>
       <c r="AF15" s="27"/>
-      <c r="AG15" s="94"/>
+      <c r="AG15" s="122"/>
       <c r="AH15" s="16">
         <v>45903</v>
       </c>
       <c r="AI15" s="23"/>
       <c r="AJ15" s="18"/>
-      <c r="AK15" s="94"/>
+      <c r="AK15" s="122"/>
       <c r="AL15" s="16">
         <v>46115</v>
       </c>
       <c r="AM15" s="23"/>
       <c r="AN15" s="19"/>
-      <c r="AO15" s="92"/>
+      <c r="AO15" s="115"/>
       <c r="AP15" s="14">
         <v>46145</v>
       </c>
       <c r="AQ15" s="21"/>
       <c r="AR15" s="59"/>
-      <c r="AS15" s="94"/>
+      <c r="AS15" s="122"/>
       <c r="AT15" s="16">
         <v>45994</v>
       </c>
       <c r="AU15" s="23"/>
       <c r="AV15" s="29"/>
     </row>
-    <row r="16" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="91"/>
+    <row r="16" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="114"/>
       <c r="B16" s="16">
         <v>45904</v>
       </c>
@@ -2583,13 +2589,13 @@
       <c r="D16" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="92"/>
+      <c r="E16" s="115"/>
       <c r="F16" s="14">
         <v>46026</v>
       </c>
       <c r="G16" s="21"/>
       <c r="H16" s="59"/>
-      <c r="I16" s="91"/>
+      <c r="I16" s="114"/>
       <c r="J16" s="16">
         <v>46057</v>
       </c>
@@ -2599,7 +2605,7 @@
       <c r="L16" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M16" s="91"/>
+      <c r="M16" s="114"/>
       <c r="N16" s="16">
         <v>46085</v>
       </c>
@@ -2607,13 +2613,13 @@
       <c r="P16" s="24">
         <v>7</v>
       </c>
-      <c r="Q16" s="94"/>
+      <c r="Q16" s="122"/>
       <c r="R16" s="14">
         <v>45934</v>
       </c>
       <c r="S16" s="15"/>
       <c r="T16" s="20"/>
-      <c r="U16" s="93" t="s">
+      <c r="U16" s="113" t="s">
         <v>21</v>
       </c>
       <c r="V16" s="16">
@@ -2623,13 +2629,13 @@
       <c r="X16" s="24">
         <v>7</v>
       </c>
-      <c r="Y16" s="91"/>
+      <c r="Y16" s="114"/>
       <c r="Z16" s="16">
         <v>45904</v>
       </c>
       <c r="AA16" s="23"/>
       <c r="AB16" s="19"/>
-      <c r="AC16" s="94" t="s">
+      <c r="AC16" s="122" t="s">
         <v>20</v>
       </c>
       <c r="AD16" s="14">
@@ -2637,19 +2643,19 @@
       </c>
       <c r="AE16" s="15"/>
       <c r="AF16" s="20"/>
-      <c r="AG16" s="94"/>
+      <c r="AG16" s="122"/>
       <c r="AH16" s="16">
         <v>45904</v>
       </c>
       <c r="AI16" s="23"/>
       <c r="AJ16" s="18"/>
-      <c r="AK16" s="94"/>
+      <c r="AK16" s="122"/>
       <c r="AL16" s="14">
         <v>46116</v>
       </c>
       <c r="AM16" s="15"/>
       <c r="AN16" s="20"/>
-      <c r="AO16" s="93" t="s">
+      <c r="AO16" s="113" t="s">
         <v>21</v>
       </c>
       <c r="AP16" s="16">
@@ -2657,15 +2663,15 @@
       </c>
       <c r="AQ16" s="23"/>
       <c r="AR16" s="19"/>
-      <c r="AS16" s="94"/>
+      <c r="AS16" s="122"/>
       <c r="AT16" s="16">
         <v>45995</v>
       </c>
       <c r="AU16" s="29"/>
       <c r="AV16" s="29"/>
     </row>
-    <row r="17" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="91"/>
+    <row r="17" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="114"/>
       <c r="B17" s="16">
         <v>45905</v>
       </c>
@@ -2675,7 +2681,7 @@
       <c r="D17" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="93" t="s">
+      <c r="E17" s="113" t="s">
         <v>65</v>
       </c>
       <c r="F17" s="16">
@@ -2687,7 +2693,7 @@
       <c r="H17" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I17" s="91"/>
+      <c r="I17" s="114"/>
       <c r="J17" s="16">
         <v>46058</v>
       </c>
@@ -2697,7 +2703,7 @@
       <c r="L17" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M17" s="91"/>
+      <c r="M17" s="114"/>
       <c r="N17" s="16">
         <v>46086</v>
       </c>
@@ -2705,13 +2711,13 @@
       <c r="P17" s="24">
         <v>7</v>
       </c>
-      <c r="Q17" s="94"/>
+      <c r="Q17" s="122"/>
       <c r="R17" s="14">
         <v>45935</v>
       </c>
       <c r="S17" s="15"/>
       <c r="T17" s="20"/>
-      <c r="U17" s="91"/>
+      <c r="U17" s="114"/>
       <c r="V17" s="16">
         <v>45874</v>
       </c>
@@ -2719,51 +2725,51 @@
       <c r="X17" s="24">
         <v>7</v>
       </c>
-      <c r="Y17" s="91"/>
+      <c r="Y17" s="114"/>
       <c r="Z17" s="16">
         <v>45905</v>
       </c>
       <c r="AA17" s="23"/>
       <c r="AB17" s="19"/>
-      <c r="AC17" s="94"/>
+      <c r="AC17" s="122"/>
       <c r="AD17" s="14">
         <v>45935</v>
       </c>
       <c r="AE17" s="15"/>
       <c r="AF17" s="20"/>
-      <c r="AG17" s="94"/>
+      <c r="AG17" s="122"/>
       <c r="AH17" s="16">
         <v>45905</v>
       </c>
       <c r="AI17" s="23"/>
       <c r="AJ17" s="18"/>
-      <c r="AK17" s="94"/>
+      <c r="AK17" s="122"/>
       <c r="AL17" s="14">
         <v>46117</v>
       </c>
       <c r="AM17" s="15"/>
       <c r="AN17" s="20"/>
-      <c r="AO17" s="91"/>
+      <c r="AO17" s="114"/>
       <c r="AP17" s="16">
         <v>46147</v>
       </c>
       <c r="AQ17" s="23"/>
       <c r="AR17" s="19"/>
-      <c r="AS17" s="94"/>
+      <c r="AS17" s="122"/>
       <c r="AT17" s="16">
         <v>45996</v>
       </c>
       <c r="AU17" s="29"/>
       <c r="AV17" s="29"/>
     </row>
-    <row r="18" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="91"/>
+    <row r="18" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="114"/>
       <c r="B18" s="14">
         <v>45906</v>
       </c>
       <c r="C18" s="21"/>
       <c r="D18" s="22"/>
-      <c r="E18" s="91"/>
+      <c r="E18" s="114"/>
       <c r="F18" s="16">
         <v>46028</v>
       </c>
@@ -2773,7 +2779,7 @@
       <c r="H18" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I18" s="91"/>
+      <c r="I18" s="114"/>
       <c r="J18" s="16">
         <v>46059</v>
       </c>
@@ -2783,7 +2789,7 @@
       <c r="L18" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M18" s="91"/>
+      <c r="M18" s="114"/>
       <c r="N18" s="16">
         <v>46087</v>
       </c>
@@ -2791,7 +2797,7 @@
       <c r="P18" s="24">
         <v>7</v>
       </c>
-      <c r="Q18" s="94" t="s">
+      <c r="Q18" s="122" t="s">
         <v>22</v>
       </c>
       <c r="R18" s="14">
@@ -2799,7 +2805,7 @@
       </c>
       <c r="S18" s="21"/>
       <c r="T18" s="59"/>
-      <c r="U18" s="91"/>
+      <c r="U18" s="114"/>
       <c r="V18" s="16">
         <v>45875</v>
       </c>
@@ -2807,25 +2813,25 @@
       <c r="X18" s="24">
         <v>7</v>
       </c>
-      <c r="Y18" s="91"/>
+      <c r="Y18" s="114"/>
       <c r="Z18" s="14">
         <v>45906</v>
       </c>
       <c r="AA18" s="21"/>
       <c r="AB18" s="22"/>
-      <c r="AC18" s="94"/>
+      <c r="AC18" s="122"/>
       <c r="AD18" s="16">
         <v>45936</v>
       </c>
       <c r="AE18" s="29"/>
       <c r="AF18" s="31"/>
-      <c r="AG18" s="94"/>
+      <c r="AG18" s="122"/>
       <c r="AH18" s="14">
         <v>45906</v>
       </c>
       <c r="AI18" s="21"/>
       <c r="AJ18" s="22"/>
-      <c r="AK18" s="94" t="s">
+      <c r="AK18" s="122" t="s">
         <v>22</v>
       </c>
       <c r="AL18" s="14">
@@ -2833,27 +2839,27 @@
       </c>
       <c r="AM18" s="21"/>
       <c r="AN18" s="59"/>
-      <c r="AO18" s="91"/>
+      <c r="AO18" s="114"/>
       <c r="AP18" s="16">
         <v>46148</v>
       </c>
       <c r="AQ18" s="23"/>
       <c r="AR18" s="19"/>
-      <c r="AS18" s="94"/>
+      <c r="AS18" s="122"/>
       <c r="AT18" s="14">
         <v>45997</v>
       </c>
       <c r="AU18" s="15"/>
       <c r="AV18" s="26"/>
     </row>
-    <row r="19" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="92"/>
+    <row r="19" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="115"/>
       <c r="B19" s="14">
         <v>45907</v>
       </c>
       <c r="C19" s="15"/>
       <c r="D19" s="20"/>
-      <c r="E19" s="91"/>
+      <c r="E19" s="114"/>
       <c r="F19" s="16">
         <v>46029</v>
       </c>
@@ -2863,19 +2869,19 @@
       <c r="H19" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I19" s="91"/>
+      <c r="I19" s="114"/>
       <c r="J19" s="14">
         <v>46060</v>
       </c>
       <c r="K19" s="15"/>
       <c r="L19" s="20"/>
-      <c r="M19" s="91"/>
+      <c r="M19" s="114"/>
       <c r="N19" s="14">
         <v>46088</v>
       </c>
       <c r="O19" s="15"/>
       <c r="P19" s="20"/>
-      <c r="Q19" s="94"/>
+      <c r="Q19" s="122"/>
       <c r="R19" s="16">
         <v>45937</v>
       </c>
@@ -2883,7 +2889,7 @@
       <c r="T19" s="24">
         <v>7</v>
       </c>
-      <c r="U19" s="91"/>
+      <c r="U19" s="114"/>
       <c r="V19" s="16">
         <v>45876</v>
       </c>
@@ -2891,45 +2897,45 @@
       <c r="X19" s="24">
         <v>7</v>
       </c>
-      <c r="Y19" s="92"/>
+      <c r="Y19" s="115"/>
       <c r="Z19" s="14">
         <v>45907</v>
       </c>
       <c r="AA19" s="15"/>
       <c r="AB19" s="20"/>
-      <c r="AC19" s="94"/>
+      <c r="AC19" s="122"/>
       <c r="AD19" s="16">
         <v>45937</v>
       </c>
       <c r="AE19" s="29"/>
       <c r="AF19" s="27"/>
-      <c r="AG19" s="94"/>
+      <c r="AG19" s="122"/>
       <c r="AH19" s="14">
         <v>45907</v>
       </c>
       <c r="AI19" s="15"/>
       <c r="AJ19" s="20"/>
-      <c r="AK19" s="94"/>
+      <c r="AK19" s="122"/>
       <c r="AL19" s="16">
         <v>46119</v>
       </c>
       <c r="AM19" s="23"/>
       <c r="AN19" s="19"/>
-      <c r="AO19" s="91"/>
+      <c r="AO19" s="114"/>
       <c r="AP19" s="16">
         <v>46149</v>
       </c>
       <c r="AQ19" s="23"/>
       <c r="AR19" s="19"/>
-      <c r="AS19" s="94"/>
+      <c r="AS19" s="122"/>
       <c r="AT19" s="14">
         <v>45998</v>
       </c>
       <c r="AU19" s="15"/>
       <c r="AV19" s="15"/>
     </row>
-    <row r="20" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="91" t="s">
+    <row r="20" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="114" t="s">
         <v>24</v>
       </c>
       <c r="B20" s="16">
@@ -2941,7 +2947,7 @@
       <c r="D20" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="91"/>
+      <c r="E20" s="114"/>
       <c r="F20" s="16">
         <v>46030</v>
       </c>
@@ -2951,19 +2957,19 @@
       <c r="H20" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="I20" s="92"/>
+      <c r="I20" s="115"/>
       <c r="J20" s="14">
         <v>46061</v>
       </c>
       <c r="K20" s="21"/>
       <c r="L20" s="20"/>
-      <c r="M20" s="92"/>
+      <c r="M20" s="115"/>
       <c r="N20" s="14">
         <v>46089</v>
       </c>
       <c r="O20" s="21"/>
       <c r="P20" s="59"/>
-      <c r="Q20" s="94"/>
+      <c r="Q20" s="122"/>
       <c r="R20" s="16">
         <v>45938</v>
       </c>
@@ -2971,13 +2977,13 @@
       <c r="T20" s="24">
         <v>7</v>
       </c>
-      <c r="U20" s="91"/>
+      <c r="U20" s="114"/>
       <c r="V20" s="14">
         <v>45877</v>
       </c>
       <c r="W20" s="21"/>
       <c r="X20" s="20"/>
-      <c r="Y20" s="91" t="s">
+      <c r="Y20" s="114" t="s">
         <v>77</v>
       </c>
       <c r="Z20" s="16">
@@ -2985,13 +2991,13 @@
       </c>
       <c r="AA20" s="23"/>
       <c r="AB20" s="19"/>
-      <c r="AC20" s="94"/>
+      <c r="AC20" s="122"/>
       <c r="AD20" s="16">
         <v>45938</v>
       </c>
       <c r="AE20" s="29"/>
       <c r="AF20" s="27"/>
-      <c r="AG20" s="94" t="s">
+      <c r="AG20" s="122" t="s">
         <v>23</v>
       </c>
       <c r="AH20" s="16">
@@ -2999,19 +3005,19 @@
       </c>
       <c r="AI20" s="29"/>
       <c r="AJ20" s="31"/>
-      <c r="AK20" s="94"/>
+      <c r="AK20" s="122"/>
       <c r="AL20" s="16">
         <v>46120</v>
       </c>
       <c r="AM20" s="23"/>
       <c r="AN20" s="19"/>
-      <c r="AO20" s="91"/>
+      <c r="AO20" s="114"/>
       <c r="AP20" s="14">
         <v>46150</v>
       </c>
       <c r="AQ20" s="15"/>
       <c r="AR20" s="59"/>
-      <c r="AS20" s="94" t="s">
+      <c r="AS20" s="122" t="s">
         <v>24</v>
       </c>
       <c r="AT20" s="16">
@@ -3020,8 +3026,8 @@
       <c r="AU20" s="29"/>
       <c r="AV20" s="29"/>
     </row>
-    <row r="21" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="91"/>
+    <row r="21" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="114"/>
       <c r="B21" s="16">
         <v>45909</v>
       </c>
@@ -3031,7 +3037,7 @@
       <c r="D21" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="E21" s="91"/>
+      <c r="E21" s="114"/>
       <c r="F21" s="16">
         <v>46031</v>
       </c>
@@ -3041,7 +3047,7 @@
       <c r="H21" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I21" s="93" t="s">
+      <c r="I21" s="113" t="s">
         <v>70</v>
       </c>
       <c r="J21" s="16">
@@ -3053,7 +3059,7 @@
       <c r="L21" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M21" s="93" t="s">
+      <c r="M21" s="113" t="s">
         <v>25</v>
       </c>
       <c r="N21" s="16">
@@ -3065,7 +3071,7 @@
       <c r="P21" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Q21" s="94"/>
+      <c r="Q21" s="122"/>
       <c r="R21" s="16">
         <v>45939</v>
       </c>
@@ -3073,51 +3079,51 @@
       <c r="T21" s="24">
         <v>7</v>
       </c>
-      <c r="U21" s="91"/>
+      <c r="U21" s="114"/>
       <c r="V21" s="14">
         <v>45878</v>
       </c>
       <c r="W21" s="15"/>
       <c r="X21" s="20"/>
-      <c r="Y21" s="91"/>
+      <c r="Y21" s="114"/>
       <c r="Z21" s="16">
         <v>45909</v>
       </c>
       <c r="AA21" s="23"/>
       <c r="AB21" s="19"/>
-      <c r="AC21" s="94"/>
+      <c r="AC21" s="122"/>
       <c r="AD21" s="16">
         <v>45939</v>
       </c>
       <c r="AE21" s="29"/>
       <c r="AF21" s="27"/>
-      <c r="AG21" s="94"/>
+      <c r="AG21" s="122"/>
       <c r="AH21" s="16">
         <v>45909</v>
       </c>
       <c r="AI21" s="23"/>
       <c r="AJ21" s="18"/>
-      <c r="AK21" s="94"/>
+      <c r="AK21" s="122"/>
       <c r="AL21" s="16">
         <v>46121</v>
       </c>
       <c r="AM21" s="23"/>
       <c r="AN21" s="19"/>
-      <c r="AO21" s="91"/>
+      <c r="AO21" s="114"/>
       <c r="AP21" s="14">
         <v>46151</v>
       </c>
       <c r="AQ21" s="21"/>
       <c r="AR21" s="22"/>
-      <c r="AS21" s="94"/>
+      <c r="AS21" s="122"/>
       <c r="AT21" s="16">
         <v>46000</v>
       </c>
       <c r="AU21" s="29"/>
       <c r="AV21" s="29"/>
     </row>
-    <row r="22" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="91"/>
+    <row r="22" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="114"/>
       <c r="B22" s="16">
         <v>45910</v>
       </c>
@@ -3127,13 +3133,13 @@
       <c r="D22" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="91"/>
+      <c r="E22" s="114"/>
       <c r="F22" s="14">
         <v>46032</v>
       </c>
       <c r="G22" s="21"/>
       <c r="H22" s="59"/>
-      <c r="I22" s="91"/>
+      <c r="I22" s="114"/>
       <c r="J22" s="16">
         <v>46063</v>
       </c>
@@ -3143,7 +3149,7 @@
       <c r="L22" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M22" s="91"/>
+      <c r="M22" s="114"/>
       <c r="N22" s="16">
         <v>46091</v>
       </c>
@@ -3153,7 +3159,7 @@
       <c r="P22" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Q22" s="94"/>
+      <c r="Q22" s="122"/>
       <c r="R22" s="16">
         <v>45940</v>
       </c>
@@ -3161,51 +3167,51 @@
       <c r="T22" s="24">
         <v>7</v>
       </c>
-      <c r="U22" s="92"/>
+      <c r="U22" s="115"/>
       <c r="V22" s="14">
         <v>45879</v>
       </c>
       <c r="W22" s="15"/>
       <c r="X22" s="20"/>
-      <c r="Y22" s="91"/>
+      <c r="Y22" s="114"/>
       <c r="Z22" s="16">
         <v>45910</v>
       </c>
       <c r="AA22" s="23"/>
       <c r="AB22" s="19"/>
-      <c r="AC22" s="94"/>
+      <c r="AC22" s="122"/>
       <c r="AD22" s="16">
         <v>45940</v>
       </c>
       <c r="AE22" s="29"/>
       <c r="AF22" s="27"/>
-      <c r="AG22" s="94"/>
+      <c r="AG22" s="122"/>
       <c r="AH22" s="16">
         <v>45910</v>
       </c>
       <c r="AI22" s="23"/>
       <c r="AJ22" s="18"/>
-      <c r="AK22" s="94"/>
+      <c r="AK22" s="122"/>
       <c r="AL22" s="16">
         <v>46122</v>
       </c>
       <c r="AM22" s="23"/>
       <c r="AN22" s="19"/>
-      <c r="AO22" s="92"/>
+      <c r="AO22" s="115"/>
       <c r="AP22" s="14">
         <v>46152</v>
       </c>
       <c r="AQ22" s="21"/>
       <c r="AR22" s="22"/>
-      <c r="AS22" s="94"/>
+      <c r="AS22" s="122"/>
       <c r="AT22" s="16">
         <v>46001</v>
       </c>
       <c r="AU22" s="29"/>
       <c r="AV22" s="29"/>
     </row>
-    <row r="23" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="91"/>
+    <row r="23" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="114"/>
       <c r="B23" s="16">
         <v>45911</v>
       </c>
@@ -3215,13 +3221,13 @@
       <c r="D23" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="E23" s="92"/>
+      <c r="E23" s="115"/>
       <c r="F23" s="14">
         <v>46033</v>
       </c>
       <c r="G23" s="21"/>
       <c r="H23" s="59"/>
-      <c r="I23" s="91"/>
+      <c r="I23" s="114"/>
       <c r="J23" s="16">
         <v>46064</v>
       </c>
@@ -3231,7 +3237,7 @@
       <c r="L23" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M23" s="91"/>
+      <c r="M23" s="114"/>
       <c r="N23" s="16">
         <v>46092</v>
       </c>
@@ -3241,13 +3247,13 @@
       <c r="P23" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Q23" s="94"/>
+      <c r="Q23" s="122"/>
       <c r="R23" s="14">
         <v>45941</v>
       </c>
       <c r="S23" s="15"/>
       <c r="T23" s="20"/>
-      <c r="U23" s="93" t="s">
+      <c r="U23" s="113" t="s">
         <v>27</v>
       </c>
       <c r="V23" s="16">
@@ -3257,13 +3263,13 @@
       <c r="X23" s="24">
         <v>7</v>
       </c>
-      <c r="Y23" s="91"/>
+      <c r="Y23" s="114"/>
       <c r="Z23" s="16">
         <v>45911</v>
       </c>
       <c r="AA23" s="23"/>
       <c r="AB23" s="19"/>
-      <c r="AC23" s="94" t="s">
+      <c r="AC23" s="122" t="s">
         <v>26</v>
       </c>
       <c r="AD23" s="14">
@@ -3271,19 +3277,19 @@
       </c>
       <c r="AE23" s="15"/>
       <c r="AF23" s="20"/>
-      <c r="AG23" s="94"/>
+      <c r="AG23" s="122"/>
       <c r="AH23" s="16">
         <v>45911</v>
       </c>
       <c r="AI23" s="23"/>
       <c r="AJ23" s="18"/>
-      <c r="AK23" s="94"/>
+      <c r="AK23" s="122"/>
       <c r="AL23" s="14">
         <v>46123</v>
       </c>
       <c r="AM23" s="15"/>
       <c r="AN23" s="20"/>
-      <c r="AO23" s="93" t="s">
+      <c r="AO23" s="113" t="s">
         <v>27</v>
       </c>
       <c r="AP23" s="16">
@@ -3291,15 +3297,15 @@
       </c>
       <c r="AQ23" s="23"/>
       <c r="AR23" s="19"/>
-      <c r="AS23" s="94"/>
+      <c r="AS23" s="122"/>
       <c r="AT23" s="16">
         <v>46002</v>
       </c>
       <c r="AU23" s="29"/>
       <c r="AV23" s="29"/>
     </row>
-    <row r="24" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="91"/>
+    <row r="24" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="114"/>
       <c r="B24" s="16">
         <v>45912</v>
       </c>
@@ -3309,7 +3315,7 @@
       <c r="D24" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E24" s="93" t="s">
+      <c r="E24" s="113" t="s">
         <v>66</v>
       </c>
       <c r="F24" s="16">
@@ -3318,10 +3324,10 @@
       <c r="G24" s="17">
         <v>7</v>
       </c>
-      <c r="H24" s="122" t="s">
+      <c r="H24" s="91" t="s">
         <v>49</v>
       </c>
-      <c r="I24" s="91"/>
+      <c r="I24" s="114"/>
       <c r="J24" s="16">
         <v>46065</v>
       </c>
@@ -3331,7 +3337,7 @@
       <c r="L24" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M24" s="91"/>
+      <c r="M24" s="114"/>
       <c r="N24" s="16">
         <v>46093</v>
       </c>
@@ -3341,13 +3347,13 @@
       <c r="P24" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Q24" s="94"/>
+      <c r="Q24" s="122"/>
       <c r="R24" s="14">
         <v>45942</v>
       </c>
       <c r="S24" s="15"/>
       <c r="T24" s="20"/>
-      <c r="U24" s="91"/>
+      <c r="U24" s="114"/>
       <c r="V24" s="16">
         <v>45881</v>
       </c>
@@ -3355,61 +3361,61 @@
       <c r="X24" s="24">
         <v>7</v>
       </c>
-      <c r="Y24" s="91"/>
+      <c r="Y24" s="114"/>
       <c r="Z24" s="16">
         <v>45912</v>
       </c>
       <c r="AA24" s="23"/>
       <c r="AB24" s="19"/>
-      <c r="AC24" s="94"/>
+      <c r="AC24" s="122"/>
       <c r="AD24" s="14">
         <v>45942</v>
       </c>
       <c r="AE24" s="15"/>
       <c r="AF24" s="20"/>
-      <c r="AG24" s="94"/>
+      <c r="AG24" s="122"/>
       <c r="AH24" s="16">
         <v>45912</v>
       </c>
       <c r="AI24" s="23"/>
       <c r="AJ24" s="18"/>
-      <c r="AK24" s="94"/>
+      <c r="AK24" s="122"/>
       <c r="AL24" s="14">
         <v>46124</v>
       </c>
       <c r="AM24" s="15"/>
       <c r="AN24" s="20"/>
-      <c r="AO24" s="91"/>
+      <c r="AO24" s="114"/>
       <c r="AP24" s="16">
         <v>46154</v>
       </c>
       <c r="AQ24" s="23"/>
       <c r="AR24" s="19"/>
-      <c r="AS24" s="94"/>
+      <c r="AS24" s="122"/>
       <c r="AT24" s="16">
         <v>46003</v>
       </c>
       <c r="AU24" s="29"/>
       <c r="AV24" s="29"/>
     </row>
-    <row r="25" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="91"/>
+    <row r="25" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="114"/>
       <c r="B25" s="14">
         <v>45913</v>
       </c>
       <c r="C25" s="21"/>
       <c r="D25" s="22"/>
-      <c r="E25" s="91"/>
+      <c r="E25" s="114"/>
       <c r="F25" s="16">
         <v>46035</v>
       </c>
       <c r="G25" s="17">
         <v>7</v>
       </c>
-      <c r="H25" s="122" t="s">
+      <c r="H25" s="91" t="s">
         <v>49</v>
       </c>
-      <c r="I25" s="91"/>
+      <c r="I25" s="114"/>
       <c r="J25" s="16">
         <v>46066</v>
       </c>
@@ -3419,7 +3425,7 @@
       <c r="L25" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M25" s="91"/>
+      <c r="M25" s="114"/>
       <c r="N25" s="16">
         <v>46094</v>
       </c>
@@ -3429,7 +3435,7 @@
       <c r="P25" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Q25" s="94" t="s">
+      <c r="Q25" s="122" t="s">
         <v>28</v>
       </c>
       <c r="R25" s="72">
@@ -3441,7 +3447,7 @@
       <c r="T25" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U25" s="91"/>
+      <c r="U25" s="114"/>
       <c r="V25" s="16">
         <v>45882</v>
       </c>
@@ -3449,25 +3455,25 @@
       <c r="X25" s="24">
         <v>7</v>
       </c>
-      <c r="Y25" s="91"/>
+      <c r="Y25" s="114"/>
       <c r="Z25" s="14">
         <v>45913</v>
       </c>
       <c r="AA25" s="21"/>
       <c r="AB25" s="22"/>
-      <c r="AC25" s="94"/>
+      <c r="AC25" s="122"/>
       <c r="AD25" s="16">
         <v>45943</v>
       </c>
       <c r="AE25" s="29"/>
       <c r="AF25" s="27"/>
-      <c r="AG25" s="94"/>
+      <c r="AG25" s="122"/>
       <c r="AH25" s="14">
         <v>45913</v>
       </c>
       <c r="AI25" s="21"/>
       <c r="AJ25" s="22"/>
-      <c r="AK25" s="94" t="s">
+      <c r="AK25" s="122" t="s">
         <v>28</v>
       </c>
       <c r="AL25" s="61">
@@ -3475,27 +3481,27 @@
       </c>
       <c r="AM25" s="23"/>
       <c r="AN25" s="27"/>
-      <c r="AO25" s="91"/>
+      <c r="AO25" s="114"/>
       <c r="AP25" s="16">
         <v>46155</v>
       </c>
       <c r="AQ25" s="23"/>
       <c r="AR25" s="19"/>
-      <c r="AS25" s="94"/>
+      <c r="AS25" s="122"/>
       <c r="AT25" s="14">
         <v>46004</v>
       </c>
       <c r="AU25" s="15"/>
       <c r="AV25" s="15"/>
     </row>
-    <row r="26" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="92"/>
+    <row r="26" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="115"/>
       <c r="B26" s="14">
         <v>45914</v>
       </c>
       <c r="C26" s="15"/>
       <c r="D26" s="20"/>
-      <c r="E26" s="91"/>
+      <c r="E26" s="114"/>
       <c r="F26" s="16">
         <v>46036</v>
       </c>
@@ -3505,19 +3511,19 @@
       <c r="H26" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="I26" s="91"/>
+      <c r="I26" s="114"/>
       <c r="J26" s="14">
         <v>46067</v>
       </c>
       <c r="K26" s="15"/>
       <c r="L26" s="22"/>
-      <c r="M26" s="91"/>
+      <c r="M26" s="114"/>
       <c r="N26" s="14">
         <v>46095</v>
       </c>
       <c r="O26" s="15"/>
       <c r="P26" s="20"/>
-      <c r="Q26" s="94"/>
+      <c r="Q26" s="122"/>
       <c r="R26" s="72">
         <v>45944</v>
       </c>
@@ -3527,51 +3533,51 @@
       <c r="T26" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U26" s="91"/>
+      <c r="U26" s="114"/>
       <c r="V26" s="14">
         <v>45883</v>
       </c>
       <c r="W26" s="15"/>
       <c r="X26" s="22"/>
-      <c r="Y26" s="92"/>
+      <c r="Y26" s="115"/>
       <c r="Z26" s="14">
         <v>45914</v>
       </c>
       <c r="AA26" s="15"/>
       <c r="AB26" s="20"/>
-      <c r="AC26" s="94"/>
+      <c r="AC26" s="122"/>
       <c r="AD26" s="16">
         <v>45944</v>
       </c>
       <c r="AE26" s="29"/>
       <c r="AF26" s="27"/>
-      <c r="AG26" s="94"/>
+      <c r="AG26" s="122"/>
       <c r="AH26" s="14">
         <v>45914</v>
       </c>
       <c r="AI26" s="15"/>
       <c r="AJ26" s="20"/>
-      <c r="AK26" s="94"/>
+      <c r="AK26" s="122"/>
       <c r="AL26" s="61">
         <v>46126</v>
       </c>
       <c r="AM26" s="23"/>
       <c r="AN26" s="27"/>
-      <c r="AO26" s="91"/>
+      <c r="AO26" s="114"/>
       <c r="AP26" s="14">
         <v>46156</v>
       </c>
       <c r="AQ26" s="21"/>
       <c r="AR26" s="59"/>
-      <c r="AS26" s="94"/>
+      <c r="AS26" s="122"/>
       <c r="AT26" s="14">
         <v>46005</v>
       </c>
       <c r="AU26" s="15"/>
       <c r="AV26" s="15"/>
     </row>
-    <row r="27" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="93" t="s">
+    <row r="27" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="113" t="s">
         <v>30</v>
       </c>
       <c r="B27" s="16">
@@ -3583,7 +3589,7 @@
       <c r="D27" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="91"/>
+      <c r="E27" s="114"/>
       <c r="F27" s="16">
         <v>46037</v>
       </c>
@@ -3593,19 +3599,19 @@
       <c r="H27" s="73" t="s">
         <v>53</v>
       </c>
-      <c r="I27" s="92"/>
+      <c r="I27" s="115"/>
       <c r="J27" s="14">
         <v>46068</v>
       </c>
       <c r="K27" s="21"/>
       <c r="L27" s="20"/>
-      <c r="M27" s="92"/>
+      <c r="M27" s="115"/>
       <c r="N27" s="14">
         <v>46096</v>
       </c>
       <c r="O27" s="21"/>
       <c r="P27" s="20"/>
-      <c r="Q27" s="94"/>
+      <c r="Q27" s="122"/>
       <c r="R27" s="72">
         <v>45945</v>
       </c>
@@ -3615,7 +3621,7 @@
       <c r="T27" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U27" s="91"/>
+      <c r="U27" s="114"/>
       <c r="V27" s="16">
         <v>45884</v>
       </c>
@@ -3623,7 +3629,7 @@
       <c r="X27" s="24">
         <v>7</v>
       </c>
-      <c r="Y27" s="93" t="s">
+      <c r="Y27" s="113" t="s">
         <v>78</v>
       </c>
       <c r="Z27" s="16">
@@ -3631,13 +3637,13 @@
       </c>
       <c r="AA27" s="23"/>
       <c r="AB27" s="19"/>
-      <c r="AC27" s="94"/>
+      <c r="AC27" s="122"/>
       <c r="AD27" s="16">
         <v>45945</v>
       </c>
       <c r="AE27" s="29"/>
       <c r="AF27" s="27"/>
-      <c r="AG27" s="94" t="s">
+      <c r="AG27" s="122" t="s">
         <v>29</v>
       </c>
       <c r="AH27" s="16">
@@ -3645,19 +3651,19 @@
       </c>
       <c r="AI27" s="29"/>
       <c r="AJ27" s="27"/>
-      <c r="AK27" s="94"/>
+      <c r="AK27" s="122"/>
       <c r="AL27" s="61">
         <v>46127</v>
       </c>
       <c r="AM27" s="23"/>
       <c r="AN27" s="27"/>
-      <c r="AO27" s="91"/>
+      <c r="AO27" s="114"/>
       <c r="AP27" s="16">
         <v>46157</v>
       </c>
       <c r="AQ27" s="23"/>
       <c r="AR27" s="19"/>
-      <c r="AS27" s="94" t="s">
+      <c r="AS27" s="122" t="s">
         <v>30</v>
       </c>
       <c r="AT27" s="16">
@@ -3666,8 +3672,8 @@
       <c r="AU27" s="29"/>
       <c r="AV27" s="29"/>
     </row>
-    <row r="28" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="91"/>
+    <row r="28" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="114"/>
       <c r="B28" s="16">
         <v>45916</v>
       </c>
@@ -3677,7 +3683,7 @@
       <c r="D28" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E28" s="91"/>
+      <c r="E28" s="114"/>
       <c r="F28" s="16">
         <v>46038</v>
       </c>
@@ -3687,7 +3693,7 @@
       <c r="H28" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I28" s="93" t="s">
+      <c r="I28" s="113" t="s">
         <v>71</v>
       </c>
       <c r="J28" s="61">
@@ -3699,7 +3705,7 @@
       <c r="L28" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M28" s="93" t="s">
+      <c r="M28" s="113" t="s">
         <v>31</v>
       </c>
       <c r="N28" s="16">
@@ -3711,7 +3717,7 @@
       <c r="P28" s="88" t="s">
         <v>91</v>
       </c>
-      <c r="Q28" s="94"/>
+      <c r="Q28" s="122"/>
       <c r="R28" s="72">
         <v>45946</v>
       </c>
@@ -3721,51 +3727,51 @@
       <c r="T28" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U28" s="91"/>
+      <c r="U28" s="114"/>
       <c r="V28" s="14">
         <v>45885</v>
       </c>
       <c r="W28" s="15"/>
       <c r="X28" s="20"/>
-      <c r="Y28" s="91"/>
+      <c r="Y28" s="114"/>
       <c r="Z28" s="16">
         <v>45916</v>
       </c>
       <c r="AA28" s="23"/>
       <c r="AB28" s="19"/>
-      <c r="AC28" s="94"/>
+      <c r="AC28" s="122"/>
       <c r="AD28" s="16">
         <v>45946</v>
       </c>
       <c r="AE28" s="29"/>
       <c r="AF28" s="27"/>
-      <c r="AG28" s="94"/>
+      <c r="AG28" s="122"/>
       <c r="AH28" s="16">
         <v>45916</v>
       </c>
       <c r="AI28" s="29"/>
       <c r="AJ28" s="27"/>
-      <c r="AK28" s="94"/>
+      <c r="AK28" s="122"/>
       <c r="AL28" s="61">
         <v>46128</v>
       </c>
       <c r="AM28" s="23"/>
       <c r="AN28" s="27"/>
-      <c r="AO28" s="91"/>
+      <c r="AO28" s="114"/>
       <c r="AP28" s="14">
         <v>46158</v>
       </c>
       <c r="AQ28" s="15"/>
       <c r="AR28" s="20"/>
-      <c r="AS28" s="94"/>
+      <c r="AS28" s="122"/>
       <c r="AT28" s="16">
         <v>46007</v>
       </c>
       <c r="AU28" s="29"/>
       <c r="AV28" s="29"/>
     </row>
-    <row r="29" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="91"/>
+    <row r="29" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="114"/>
       <c r="B29" s="16">
         <v>45917</v>
       </c>
@@ -3775,13 +3781,13 @@
       <c r="D29" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E29" s="91"/>
+      <c r="E29" s="114"/>
       <c r="F29" s="14">
         <v>46039</v>
       </c>
       <c r="G29" s="21"/>
       <c r="H29" s="59"/>
-      <c r="I29" s="91"/>
+      <c r="I29" s="114"/>
       <c r="J29" s="61">
         <v>46070</v>
       </c>
@@ -3791,7 +3797,7 @@
       <c r="L29" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M29" s="91"/>
+      <c r="M29" s="114"/>
       <c r="N29" s="16">
         <v>46098</v>
       </c>
@@ -3801,7 +3807,7 @@
       <c r="P29" s="88" t="s">
         <v>91</v>
       </c>
-      <c r="Q29" s="94"/>
+      <c r="Q29" s="122"/>
       <c r="R29" s="72">
         <v>45947</v>
       </c>
@@ -3811,51 +3817,51 @@
       <c r="T29" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U29" s="92"/>
+      <c r="U29" s="115"/>
       <c r="V29" s="14">
         <v>45886</v>
       </c>
       <c r="W29" s="21"/>
       <c r="X29" s="22"/>
-      <c r="Y29" s="91"/>
+      <c r="Y29" s="114"/>
       <c r="Z29" s="16">
         <v>45917</v>
       </c>
       <c r="AA29" s="23"/>
       <c r="AB29" s="19"/>
-      <c r="AC29" s="94"/>
+      <c r="AC29" s="122"/>
       <c r="AD29" s="16">
         <v>45947</v>
       </c>
       <c r="AE29" s="29"/>
       <c r="AF29" s="27"/>
-      <c r="AG29" s="94"/>
+      <c r="AG29" s="122"/>
       <c r="AH29" s="16">
         <v>45917</v>
       </c>
       <c r="AI29" s="29"/>
       <c r="AJ29" s="27"/>
-      <c r="AK29" s="94"/>
+      <c r="AK29" s="122"/>
       <c r="AL29" s="61">
         <v>46129</v>
       </c>
       <c r="AM29" s="23"/>
       <c r="AN29" s="27"/>
-      <c r="AO29" s="92"/>
+      <c r="AO29" s="115"/>
       <c r="AP29" s="14">
         <v>46159</v>
       </c>
       <c r="AQ29" s="21"/>
       <c r="AR29" s="59"/>
-      <c r="AS29" s="94"/>
+      <c r="AS29" s="122"/>
       <c r="AT29" s="16">
         <v>46008</v>
       </c>
       <c r="AU29" s="29"/>
       <c r="AV29" s="29"/>
     </row>
-    <row r="30" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="91"/>
+    <row r="30" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="114"/>
       <c r="B30" s="16">
         <v>45918</v>
       </c>
@@ -3865,13 +3871,13 @@
       <c r="D30" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E30" s="92"/>
+      <c r="E30" s="115"/>
       <c r="F30" s="14">
         <v>46040</v>
       </c>
       <c r="G30" s="21"/>
       <c r="H30" s="59"/>
-      <c r="I30" s="91"/>
+      <c r="I30" s="114"/>
       <c r="J30" s="61">
         <v>46071</v>
       </c>
@@ -3881,7 +3887,7 @@
       <c r="L30" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M30" s="91"/>
+      <c r="M30" s="114"/>
       <c r="N30" s="16">
         <v>46099</v>
       </c>
@@ -3891,13 +3897,13 @@
       <c r="P30" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="Q30" s="94"/>
+      <c r="Q30" s="122"/>
       <c r="R30" s="14">
         <v>45948</v>
       </c>
       <c r="S30" s="15"/>
       <c r="T30" s="20"/>
-      <c r="U30" s="93" t="s">
+      <c r="U30" s="113" t="s">
         <v>33</v>
       </c>
       <c r="V30" s="16">
@@ -3909,13 +3915,13 @@
       <c r="X30" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Y30" s="91"/>
+      <c r="Y30" s="114"/>
       <c r="Z30" s="16">
         <v>45918</v>
       </c>
       <c r="AA30" s="23"/>
       <c r="AB30" s="19"/>
-      <c r="AC30" s="94" t="s">
+      <c r="AC30" s="122" t="s">
         <v>32</v>
       </c>
       <c r="AD30" s="14">
@@ -3923,19 +3929,19 @@
       </c>
       <c r="AE30" s="15"/>
       <c r="AF30" s="20"/>
-      <c r="AG30" s="94"/>
+      <c r="AG30" s="122"/>
       <c r="AH30" s="16">
         <v>45918</v>
       </c>
       <c r="AI30" s="29"/>
       <c r="AJ30" s="27"/>
-      <c r="AK30" s="94"/>
+      <c r="AK30" s="122"/>
       <c r="AL30" s="14">
         <v>46130</v>
       </c>
       <c r="AM30" s="15"/>
       <c r="AN30" s="20"/>
-      <c r="AO30" s="93" t="s">
+      <c r="AO30" s="113" t="s">
         <v>33</v>
       </c>
       <c r="AP30" s="16">
@@ -3943,15 +3949,15 @@
       </c>
       <c r="AQ30" s="23"/>
       <c r="AR30" s="19"/>
-      <c r="AS30" s="94"/>
+      <c r="AS30" s="122"/>
       <c r="AT30" s="16">
         <v>46009</v>
       </c>
       <c r="AU30" s="29"/>
       <c r="AV30" s="29"/>
     </row>
-    <row r="31" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="91"/>
+    <row r="31" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="114"/>
       <c r="B31" s="16">
         <v>45919</v>
       </c>
@@ -3961,7 +3967,7 @@
       <c r="D31" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E31" s="93" t="s">
+      <c r="E31" s="113" t="s">
         <v>67</v>
       </c>
       <c r="F31" s="16">
@@ -3973,7 +3979,7 @@
       <c r="H31" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="I31" s="91"/>
+      <c r="I31" s="114"/>
       <c r="J31" s="61">
         <v>46072</v>
       </c>
@@ -3983,7 +3989,7 @@
       <c r="L31" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M31" s="91"/>
+      <c r="M31" s="114"/>
       <c r="N31" s="16">
         <v>46100</v>
       </c>
@@ -3993,13 +3999,13 @@
       <c r="P31" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="Q31" s="94"/>
+      <c r="Q31" s="122"/>
       <c r="R31" s="14">
         <v>45949</v>
       </c>
       <c r="S31" s="15"/>
       <c r="T31" s="20"/>
-      <c r="U31" s="91"/>
+      <c r="U31" s="114"/>
       <c r="V31" s="16">
         <v>45888</v>
       </c>
@@ -4009,51 +4015,51 @@
       <c r="X31" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Y31" s="91"/>
+      <c r="Y31" s="114"/>
       <c r="Z31" s="16">
         <v>45919</v>
       </c>
       <c r="AA31" s="23"/>
       <c r="AB31" s="19"/>
-      <c r="AC31" s="94"/>
+      <c r="AC31" s="122"/>
       <c r="AD31" s="14">
         <v>45949</v>
       </c>
       <c r="AE31" s="15"/>
       <c r="AF31" s="20"/>
-      <c r="AG31" s="94"/>
+      <c r="AG31" s="122"/>
       <c r="AH31" s="16">
         <v>45919</v>
       </c>
       <c r="AI31" s="29"/>
       <c r="AJ31" s="27"/>
-      <c r="AK31" s="94"/>
+      <c r="AK31" s="122"/>
       <c r="AL31" s="14">
         <v>46131</v>
       </c>
       <c r="AM31" s="15"/>
       <c r="AN31" s="20"/>
-      <c r="AO31" s="91"/>
+      <c r="AO31" s="114"/>
       <c r="AP31" s="16">
         <v>46161</v>
       </c>
       <c r="AQ31" s="23"/>
       <c r="AR31" s="19"/>
-      <c r="AS31" s="94"/>
+      <c r="AS31" s="122"/>
       <c r="AT31" s="16">
         <v>46010</v>
       </c>
       <c r="AU31" s="29"/>
       <c r="AV31" s="29"/>
     </row>
-    <row r="32" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="91"/>
+    <row r="32" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="114"/>
       <c r="B32" s="14">
         <v>45920</v>
       </c>
       <c r="C32" s="15"/>
       <c r="D32" s="20"/>
-      <c r="E32" s="91"/>
+      <c r="E32" s="114"/>
       <c r="F32" s="16">
         <v>46042</v>
       </c>
@@ -4063,7 +4069,7 @@
       <c r="H32" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I32" s="91"/>
+      <c r="I32" s="114"/>
       <c r="J32" s="61">
         <v>46073</v>
       </c>
@@ -4073,7 +4079,7 @@
       <c r="L32" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="M32" s="91"/>
+      <c r="M32" s="114"/>
       <c r="N32" s="16">
         <v>46101</v>
       </c>
@@ -4083,7 +4089,7 @@
       <c r="P32" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Q32" s="94" t="s">
+      <c r="Q32" s="122" t="s">
         <v>34</v>
       </c>
       <c r="R32" s="72">
@@ -4095,7 +4101,7 @@
       <c r="T32" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U32" s="91"/>
+      <c r="U32" s="114"/>
       <c r="V32" s="16">
         <v>45889</v>
       </c>
@@ -4105,25 +4111,25 @@
       <c r="X32" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Y32" s="91"/>
+      <c r="Y32" s="114"/>
       <c r="Z32" s="14">
         <v>45920</v>
       </c>
       <c r="AA32" s="15"/>
       <c r="AB32" s="20"/>
-      <c r="AC32" s="94"/>
+      <c r="AC32" s="122"/>
       <c r="AD32" s="16">
         <v>45950</v>
       </c>
       <c r="AE32" s="29"/>
       <c r="AF32" s="27"/>
-      <c r="AG32" s="94"/>
+      <c r="AG32" s="122"/>
       <c r="AH32" s="14">
         <v>45920</v>
       </c>
       <c r="AI32" s="15"/>
       <c r="AJ32" s="20"/>
-      <c r="AK32" s="94" t="s">
+      <c r="AK32" s="122" t="s">
         <v>34</v>
       </c>
       <c r="AL32" s="61">
@@ -4131,27 +4137,27 @@
       </c>
       <c r="AM32" s="23"/>
       <c r="AN32" s="27"/>
-      <c r="AO32" s="91"/>
+      <c r="AO32" s="114"/>
       <c r="AP32" s="16">
         <v>46162</v>
       </c>
       <c r="AQ32" s="23"/>
       <c r="AR32" s="19"/>
-      <c r="AS32" s="94"/>
+      <c r="AS32" s="122"/>
       <c r="AT32" s="14">
         <v>46011</v>
       </c>
       <c r="AU32" s="15"/>
       <c r="AV32" s="15"/>
     </row>
-    <row r="33" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="92"/>
+    <row r="33" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="115"/>
       <c r="B33" s="14">
         <v>45921</v>
       </c>
       <c r="C33" s="15"/>
       <c r="D33" s="20"/>
-      <c r="E33" s="91"/>
+      <c r="E33" s="114"/>
       <c r="F33" s="16">
         <v>46043</v>
       </c>
@@ -4161,19 +4167,19 @@
       <c r="H33" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I33" s="91"/>
+      <c r="I33" s="114"/>
       <c r="J33" s="14">
         <v>46074</v>
       </c>
       <c r="K33" s="15"/>
       <c r="L33" s="20"/>
-      <c r="M33" s="91"/>
+      <c r="M33" s="114"/>
       <c r="N33" s="14">
         <v>46102</v>
       </c>
       <c r="O33" s="15"/>
       <c r="P33" s="20"/>
-      <c r="Q33" s="94"/>
+      <c r="Q33" s="122"/>
       <c r="R33" s="72">
         <v>45951</v>
       </c>
@@ -4183,7 +4189,7 @@
       <c r="T33" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U33" s="91"/>
+      <c r="U33" s="114"/>
       <c r="V33" s="16">
         <v>45890</v>
       </c>
@@ -4193,45 +4199,45 @@
       <c r="X33" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Y33" s="92"/>
+      <c r="Y33" s="115"/>
       <c r="Z33" s="14">
         <v>45921</v>
       </c>
       <c r="AA33" s="15"/>
       <c r="AB33" s="20"/>
-      <c r="AC33" s="94"/>
+      <c r="AC33" s="122"/>
       <c r="AD33" s="16">
         <v>45951</v>
       </c>
       <c r="AE33" s="29"/>
       <c r="AF33" s="27"/>
-      <c r="AG33" s="94"/>
+      <c r="AG33" s="122"/>
       <c r="AH33" s="14">
         <v>45921</v>
       </c>
       <c r="AI33" s="15"/>
       <c r="AJ33" s="20"/>
-      <c r="AK33" s="94"/>
+      <c r="AK33" s="122"/>
       <c r="AL33" s="61">
         <v>46133</v>
       </c>
       <c r="AM33" s="23"/>
       <c r="AN33" s="27"/>
-      <c r="AO33" s="91"/>
+      <c r="AO33" s="114"/>
       <c r="AP33" s="16">
         <v>46163</v>
       </c>
       <c r="AQ33" s="23"/>
       <c r="AR33" s="19"/>
-      <c r="AS33" s="94"/>
+      <c r="AS33" s="122"/>
       <c r="AT33" s="14">
         <v>46012</v>
       </c>
       <c r="AU33" s="15"/>
       <c r="AV33" s="15"/>
     </row>
-    <row r="34" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="93" t="s">
+    <row r="34" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="113" t="s">
         <v>36</v>
       </c>
       <c r="B34" s="72">
@@ -4243,7 +4249,7 @@
       <c r="D34" s="89" t="s">
         <v>50</v>
       </c>
-      <c r="E34" s="91"/>
+      <c r="E34" s="114"/>
       <c r="F34" s="16">
         <v>46044</v>
       </c>
@@ -4253,19 +4259,19 @@
       <c r="H34" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I34" s="92"/>
+      <c r="I34" s="115"/>
       <c r="J34" s="14">
         <v>46075</v>
       </c>
       <c r="K34" s="21"/>
       <c r="L34" s="20"/>
-      <c r="M34" s="92"/>
+      <c r="M34" s="115"/>
       <c r="N34" s="14">
         <v>46103</v>
       </c>
       <c r="O34" s="21"/>
       <c r="P34" s="20"/>
-      <c r="Q34" s="94"/>
+      <c r="Q34" s="122"/>
       <c r="R34" s="72">
         <v>45952</v>
       </c>
@@ -4275,7 +4281,7 @@
       <c r="T34" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U34" s="91"/>
+      <c r="U34" s="114"/>
       <c r="V34" s="16">
         <v>45891</v>
       </c>
@@ -4285,7 +4291,7 @@
       <c r="X34" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Y34" s="93" t="s">
+      <c r="Y34" s="113" t="s">
         <v>79</v>
       </c>
       <c r="Z34" s="16">
@@ -4293,13 +4299,13 @@
       </c>
       <c r="AA34" s="23"/>
       <c r="AB34" s="19"/>
-      <c r="AC34" s="94"/>
+      <c r="AC34" s="122"/>
       <c r="AD34" s="16">
         <v>45952</v>
       </c>
       <c r="AE34" s="29"/>
       <c r="AF34" s="27"/>
-      <c r="AG34" s="94" t="s">
+      <c r="AG34" s="122" t="s">
         <v>35</v>
       </c>
       <c r="AH34" s="16">
@@ -4307,19 +4313,19 @@
       </c>
       <c r="AI34" s="29"/>
       <c r="AJ34" s="27"/>
-      <c r="AK34" s="94"/>
+      <c r="AK34" s="122"/>
       <c r="AL34" s="61">
         <v>46134</v>
       </c>
       <c r="AM34" s="23"/>
       <c r="AN34" s="27"/>
-      <c r="AO34" s="91"/>
+      <c r="AO34" s="114"/>
       <c r="AP34" s="16">
         <v>46164</v>
       </c>
       <c r="AQ34" s="23"/>
       <c r="AR34" s="19"/>
-      <c r="AS34" s="94" t="s">
+      <c r="AS34" s="122" t="s">
         <v>36</v>
       </c>
       <c r="AT34" s="16">
@@ -4328,8 +4334,8 @@
       <c r="AU34" s="29"/>
       <c r="AV34" s="29"/>
     </row>
-    <row r="35" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="91"/>
+    <row r="35" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="114"/>
       <c r="B35" s="72">
         <v>45923</v>
       </c>
@@ -4339,7 +4345,7 @@
       <c r="D35" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E35" s="91"/>
+      <c r="E35" s="114"/>
       <c r="F35" s="16">
         <v>46045</v>
       </c>
@@ -4349,7 +4355,7 @@
       <c r="H35" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I35" s="93" t="s">
+      <c r="I35" s="113" t="s">
         <v>72</v>
       </c>
       <c r="J35" s="61">
@@ -4359,7 +4365,7 @@
       <c r="L35" s="24">
         <v>7</v>
       </c>
-      <c r="M35" s="93" t="s">
+      <c r="M35" s="113" t="s">
         <v>37</v>
       </c>
       <c r="N35" s="16">
@@ -4369,7 +4375,7 @@
       <c r="P35" s="24">
         <v>7</v>
       </c>
-      <c r="Q35" s="94"/>
+      <c r="Q35" s="122"/>
       <c r="R35" s="72">
         <v>45953</v>
       </c>
@@ -4379,51 +4385,51 @@
       <c r="T35" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U35" s="91"/>
+      <c r="U35" s="114"/>
       <c r="V35" s="14">
         <v>45892</v>
       </c>
       <c r="W35" s="15"/>
       <c r="X35" s="20"/>
-      <c r="Y35" s="91"/>
+      <c r="Y35" s="114"/>
       <c r="Z35" s="16">
         <v>45923</v>
       </c>
       <c r="AA35" s="23"/>
       <c r="AB35" s="19"/>
-      <c r="AC35" s="94"/>
+      <c r="AC35" s="122"/>
       <c r="AD35" s="16">
         <v>45953</v>
       </c>
       <c r="AE35" s="29"/>
       <c r="AF35" s="27"/>
-      <c r="AG35" s="94"/>
+      <c r="AG35" s="122"/>
       <c r="AH35" s="16">
         <v>45923</v>
       </c>
       <c r="AI35" s="29"/>
       <c r="AJ35" s="27"/>
-      <c r="AK35" s="94"/>
+      <c r="AK35" s="122"/>
       <c r="AL35" s="61">
         <v>46135</v>
       </c>
       <c r="AM35" s="23"/>
       <c r="AN35" s="27"/>
-      <c r="AO35" s="91"/>
+      <c r="AO35" s="114"/>
       <c r="AP35" s="14">
         <v>46165</v>
       </c>
       <c r="AQ35" s="15"/>
       <c r="AR35" s="20"/>
-      <c r="AS35" s="94"/>
+      <c r="AS35" s="122"/>
       <c r="AT35" s="16">
         <v>46014</v>
       </c>
       <c r="AU35" s="29"/>
       <c r="AV35" s="29"/>
     </row>
-    <row r="36" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="91"/>
+    <row r="36" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="114"/>
       <c r="B36" s="72">
         <v>45924</v>
       </c>
@@ -4433,13 +4439,13 @@
       <c r="D36" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E36" s="91"/>
+      <c r="E36" s="114"/>
       <c r="F36" s="14">
         <v>46046</v>
       </c>
       <c r="G36" s="21"/>
       <c r="H36" s="20"/>
-      <c r="I36" s="91"/>
+      <c r="I36" s="114"/>
       <c r="J36" s="61">
         <v>46077</v>
       </c>
@@ -4447,7 +4453,7 @@
       <c r="L36" s="24">
         <v>7</v>
       </c>
-      <c r="M36" s="91"/>
+      <c r="M36" s="114"/>
       <c r="N36" s="16">
         <v>46105</v>
       </c>
@@ -4455,7 +4461,7 @@
       <c r="P36" s="24">
         <v>7</v>
       </c>
-      <c r="Q36" s="94"/>
+      <c r="Q36" s="122"/>
       <c r="R36" s="72">
         <v>45954</v>
       </c>
@@ -4465,63 +4471,63 @@
       <c r="T36" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="U36" s="92"/>
+      <c r="U36" s="115"/>
       <c r="V36" s="14">
         <v>45893</v>
       </c>
       <c r="W36" s="15"/>
       <c r="X36" s="20"/>
-      <c r="Y36" s="91"/>
+      <c r="Y36" s="114"/>
       <c r="Z36" s="16">
         <v>45924</v>
       </c>
       <c r="AA36" s="23"/>
       <c r="AB36" s="19"/>
-      <c r="AC36" s="94"/>
+      <c r="AC36" s="122"/>
       <c r="AD36" s="16">
         <v>45954</v>
       </c>
       <c r="AE36" s="29"/>
       <c r="AF36" s="27"/>
-      <c r="AG36" s="94"/>
+      <c r="AG36" s="122"/>
       <c r="AH36" s="16">
         <v>45924</v>
       </c>
       <c r="AI36" s="29"/>
       <c r="AJ36" s="27"/>
-      <c r="AK36" s="94"/>
+      <c r="AK36" s="122"/>
       <c r="AL36" s="61">
         <v>46136</v>
       </c>
       <c r="AM36" s="23"/>
       <c r="AN36" s="27"/>
-      <c r="AO36" s="92"/>
+      <c r="AO36" s="115"/>
       <c r="AP36" s="14">
         <v>46166</v>
       </c>
       <c r="AQ36" s="15"/>
       <c r="AR36" s="20"/>
-      <c r="AS36" s="94"/>
+      <c r="AS36" s="122"/>
       <c r="AT36" s="16">
         <v>46015</v>
       </c>
       <c r="AU36" s="29"/>
       <c r="AV36" s="29"/>
     </row>
-    <row r="37" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="91"/>
+    <row r="37" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="114"/>
       <c r="B37" s="14">
         <v>45925</v>
       </c>
       <c r="C37" s="21"/>
       <c r="D37" s="20"/>
-      <c r="E37" s="92"/>
+      <c r="E37" s="115"/>
       <c r="F37" s="14">
         <v>46047</v>
       </c>
       <c r="G37" s="21"/>
       <c r="H37" s="20"/>
-      <c r="I37" s="91"/>
+      <c r="I37" s="114"/>
       <c r="J37" s="61">
         <v>46078</v>
       </c>
@@ -4529,7 +4535,7 @@
       <c r="L37" s="24">
         <v>7</v>
       </c>
-      <c r="M37" s="91"/>
+      <c r="M37" s="114"/>
       <c r="N37" s="16">
         <v>46106</v>
       </c>
@@ -4537,13 +4543,13 @@
       <c r="P37" s="24">
         <v>7</v>
       </c>
-      <c r="Q37" s="94"/>
+      <c r="Q37" s="122"/>
       <c r="R37" s="14">
         <v>45955</v>
       </c>
       <c r="S37" s="15"/>
       <c r="T37" s="20"/>
-      <c r="U37" s="93" t="s">
+      <c r="U37" s="113" t="s">
         <v>39</v>
       </c>
       <c r="V37" s="14">
@@ -4553,13 +4559,13 @@
       <c r="X37" s="20">
         <v>7</v>
       </c>
-      <c r="Y37" s="91"/>
+      <c r="Y37" s="114"/>
       <c r="Z37" s="16">
         <v>45925</v>
       </c>
       <c r="AA37" s="23"/>
       <c r="AB37" s="27"/>
-      <c r="AC37" s="94" t="s">
+      <c r="AC37" s="122" t="s">
         <v>38</v>
       </c>
       <c r="AD37" s="14">
@@ -4567,19 +4573,19 @@
       </c>
       <c r="AE37" s="15"/>
       <c r="AF37" s="20"/>
-      <c r="AG37" s="94"/>
+      <c r="AG37" s="122"/>
       <c r="AH37" s="16">
         <v>45925</v>
       </c>
       <c r="AI37" s="29"/>
       <c r="AJ37" s="27"/>
-      <c r="AK37" s="94"/>
+      <c r="AK37" s="122"/>
       <c r="AL37" s="14">
         <v>46137</v>
       </c>
       <c r="AM37" s="15"/>
       <c r="AN37" s="20"/>
-      <c r="AO37" s="93" t="s">
+      <c r="AO37" s="113" t="s">
         <v>39</v>
       </c>
       <c r="AP37" s="14">
@@ -4587,21 +4593,21 @@
       </c>
       <c r="AQ37" s="15"/>
       <c r="AR37" s="20"/>
-      <c r="AS37" s="94"/>
+      <c r="AS37" s="122"/>
       <c r="AT37" s="14">
         <v>46016</v>
       </c>
       <c r="AU37" s="15"/>
       <c r="AV37" s="15"/>
     </row>
-    <row r="38" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="91"/>
+    <row r="38" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="114"/>
       <c r="B38" s="72">
         <v>45926</v>
       </c>
       <c r="C38" s="83"/>
       <c r="D38" s="84"/>
-      <c r="E38" s="93" t="s">
+      <c r="E38" s="113" t="s">
         <v>68</v>
       </c>
       <c r="F38" s="16">
@@ -4613,7 +4619,7 @@
       <c r="H38" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I38" s="91"/>
+      <c r="I38" s="114"/>
       <c r="J38" s="61">
         <v>46079</v>
       </c>
@@ -4621,7 +4627,7 @@
       <c r="L38" s="24">
         <v>7</v>
       </c>
-      <c r="M38" s="91"/>
+      <c r="M38" s="114"/>
       <c r="N38" s="16">
         <v>46107</v>
       </c>
@@ -4629,13 +4635,13 @@
       <c r="P38" s="24">
         <v>7</v>
       </c>
-      <c r="Q38" s="94"/>
+      <c r="Q38" s="122"/>
       <c r="R38" s="14">
         <v>45956</v>
       </c>
       <c r="S38" s="15"/>
       <c r="T38" s="20"/>
-      <c r="U38" s="91"/>
+      <c r="U38" s="114"/>
       <c r="V38" s="16">
         <v>45895</v>
       </c>
@@ -4645,51 +4651,51 @@
       <c r="X38" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Y38" s="91"/>
+      <c r="Y38" s="114"/>
       <c r="Z38" s="16">
         <v>45926</v>
       </c>
       <c r="AA38" s="23"/>
       <c r="AB38" s="27"/>
-      <c r="AC38" s="94"/>
+      <c r="AC38" s="122"/>
       <c r="AD38" s="14">
         <v>45956</v>
       </c>
       <c r="AE38" s="15"/>
       <c r="AF38" s="20"/>
-      <c r="AG38" s="94"/>
+      <c r="AG38" s="122"/>
       <c r="AH38" s="16">
         <v>45926</v>
       </c>
       <c r="AI38" s="29"/>
       <c r="AJ38" s="31"/>
-      <c r="AK38" s="94"/>
+      <c r="AK38" s="122"/>
       <c r="AL38" s="14">
         <v>46138</v>
       </c>
       <c r="AM38" s="15"/>
       <c r="AN38" s="20"/>
-      <c r="AO38" s="91"/>
+      <c r="AO38" s="114"/>
       <c r="AP38" s="16">
         <v>46168</v>
       </c>
       <c r="AQ38" s="29"/>
       <c r="AR38" s="19"/>
-      <c r="AS38" s="94"/>
+      <c r="AS38" s="122"/>
       <c r="AT38" s="16">
         <v>46017</v>
       </c>
       <c r="AU38" s="29"/>
       <c r="AV38" s="29"/>
     </row>
-    <row r="39" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="91"/>
+    <row r="39" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="114"/>
       <c r="B39" s="14">
         <v>45927</v>
       </c>
       <c r="C39" s="15"/>
       <c r="D39" s="20"/>
-      <c r="E39" s="91"/>
+      <c r="E39" s="114"/>
       <c r="F39" s="16">
         <v>46049</v>
       </c>
@@ -4699,7 +4705,7 @@
       <c r="H39" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I39" s="91"/>
+      <c r="I39" s="114"/>
       <c r="J39" s="61">
         <v>46080</v>
       </c>
@@ -4707,7 +4713,7 @@
       <c r="L39" s="24">
         <v>7</v>
       </c>
-      <c r="M39" s="91"/>
+      <c r="M39" s="114"/>
       <c r="N39" s="16">
         <v>46108</v>
       </c>
@@ -4715,7 +4721,7 @@
       <c r="P39" s="24">
         <v>7</v>
       </c>
-      <c r="Q39" s="94" t="s">
+      <c r="Q39" s="122" t="s">
         <v>14</v>
       </c>
       <c r="R39" s="16">
@@ -4725,7 +4731,7 @@
       <c r="T39" s="24">
         <v>7</v>
       </c>
-      <c r="U39" s="91"/>
+      <c r="U39" s="114"/>
       <c r="V39" s="16">
         <v>45896</v>
       </c>
@@ -4735,25 +4741,25 @@
       <c r="X39" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Y39" s="91"/>
+      <c r="Y39" s="114"/>
       <c r="Z39" s="14">
         <v>45927</v>
       </c>
       <c r="AA39" s="15"/>
       <c r="AB39" s="20"/>
-      <c r="AC39" s="94"/>
+      <c r="AC39" s="122"/>
       <c r="AD39" s="16">
         <v>45957</v>
       </c>
       <c r="AE39" s="29"/>
       <c r="AF39" s="27"/>
-      <c r="AG39" s="94"/>
+      <c r="AG39" s="122"/>
       <c r="AH39" s="14">
         <v>45927</v>
       </c>
       <c r="AI39" s="15"/>
       <c r="AJ39" s="20"/>
-      <c r="AK39" s="94" t="s">
+      <c r="AK39" s="122" t="s">
         <v>14</v>
       </c>
       <c r="AL39" s="16">
@@ -4761,27 +4767,27 @@
       </c>
       <c r="AM39" s="23"/>
       <c r="AN39" s="19"/>
-      <c r="AO39" s="91"/>
+      <c r="AO39" s="114"/>
       <c r="AP39" s="16">
         <v>46169</v>
       </c>
       <c r="AQ39" s="29"/>
       <c r="AR39" s="27"/>
-      <c r="AS39" s="94"/>
+      <c r="AS39" s="122"/>
       <c r="AT39" s="14">
         <v>46018</v>
       </c>
       <c r="AU39" s="15"/>
       <c r="AV39" s="15"/>
     </row>
-    <row r="40" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="92"/>
+    <row r="40" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="115"/>
       <c r="B40" s="14">
         <v>45928</v>
       </c>
       <c r="C40" s="15"/>
       <c r="D40" s="20"/>
-      <c r="E40" s="91"/>
+      <c r="E40" s="114"/>
       <c r="F40" s="16">
         <v>46050</v>
       </c>
@@ -4791,19 +4797,19 @@
       <c r="H40" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="I40" s="92"/>
+      <c r="I40" s="115"/>
       <c r="J40" s="14">
         <v>46081</v>
       </c>
       <c r="K40" s="21"/>
       <c r="L40" s="59"/>
-      <c r="M40" s="91"/>
+      <c r="M40" s="114"/>
       <c r="N40" s="14">
         <v>46109</v>
       </c>
       <c r="O40" s="15"/>
       <c r="P40" s="20"/>
-      <c r="Q40" s="94"/>
+      <c r="Q40" s="122"/>
       <c r="R40" s="16">
         <v>45958</v>
       </c>
@@ -4811,7 +4817,7 @@
       <c r="T40" s="24">
         <v>7</v>
       </c>
-      <c r="U40" s="91"/>
+      <c r="U40" s="114"/>
       <c r="V40" s="16">
         <v>45897</v>
       </c>
@@ -4821,45 +4827,45 @@
       <c r="X40" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="Y40" s="92"/>
+      <c r="Y40" s="115"/>
       <c r="Z40" s="14">
         <v>45928</v>
       </c>
       <c r="AA40" s="15"/>
       <c r="AB40" s="20"/>
-      <c r="AC40" s="94"/>
+      <c r="AC40" s="122"/>
       <c r="AD40" s="16">
         <v>45958</v>
       </c>
       <c r="AE40" s="29"/>
       <c r="AF40" s="27"/>
-      <c r="AG40" s="94"/>
+      <c r="AG40" s="122"/>
       <c r="AH40" s="14">
         <v>45928</v>
       </c>
       <c r="AI40" s="15"/>
       <c r="AJ40" s="20"/>
-      <c r="AK40" s="94"/>
+      <c r="AK40" s="122"/>
       <c r="AL40" s="16">
         <v>46140</v>
       </c>
       <c r="AM40" s="23"/>
       <c r="AN40" s="19"/>
-      <c r="AO40" s="91"/>
+      <c r="AO40" s="114"/>
       <c r="AP40" s="16">
         <v>46170</v>
       </c>
       <c r="AQ40" s="29"/>
       <c r="AR40" s="27"/>
-      <c r="AS40" s="94"/>
+      <c r="AS40" s="122"/>
       <c r="AT40" s="14">
         <v>46019</v>
       </c>
       <c r="AU40" s="15"/>
       <c r="AV40" s="15"/>
     </row>
-    <row r="41" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="91"/>
+    <row r="41" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="114"/>
       <c r="B41" s="72">
         <v>45929</v>
       </c>
@@ -4869,7 +4875,7 @@
       <c r="D41" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E41" s="91"/>
+      <c r="E41" s="114"/>
       <c r="F41" s="16">
         <v>46051</v>
       </c>
@@ -4883,13 +4889,13 @@
       <c r="J41" s="16"/>
       <c r="K41" s="23"/>
       <c r="L41" s="19"/>
-      <c r="M41" s="92"/>
+      <c r="M41" s="115"/>
       <c r="N41" s="14">
         <v>46110</v>
       </c>
       <c r="O41" s="21"/>
       <c r="P41" s="59"/>
-      <c r="Q41" s="94"/>
+      <c r="Q41" s="122"/>
       <c r="R41" s="16">
         <v>45959</v>
       </c>
@@ -4897,7 +4903,7 @@
       <c r="T41" s="24">
         <v>7</v>
       </c>
-      <c r="U41" s="91"/>
+      <c r="U41" s="114"/>
       <c r="V41" s="16">
         <v>45898</v>
       </c>
@@ -4907,45 +4913,45 @@
       <c r="X41" s="87" t="s">
         <v>57</v>
       </c>
-      <c r="Y41" s="91"/>
+      <c r="Y41" s="114"/>
       <c r="Z41" s="16">
         <v>45929</v>
       </c>
       <c r="AA41" s="23"/>
       <c r="AB41" s="19"/>
-      <c r="AC41" s="94"/>
+      <c r="AC41" s="122"/>
       <c r="AD41" s="16">
         <v>45959</v>
       </c>
       <c r="AE41" s="29"/>
       <c r="AF41" s="27"/>
-      <c r="AG41" s="94"/>
+      <c r="AG41" s="122"/>
       <c r="AH41" s="16">
         <v>45929</v>
       </c>
       <c r="AI41" s="29"/>
       <c r="AJ41" s="27"/>
-      <c r="AK41" s="94"/>
+      <c r="AK41" s="122"/>
       <c r="AL41" s="16">
         <v>46141</v>
       </c>
       <c r="AM41" s="23"/>
       <c r="AN41" s="19"/>
-      <c r="AO41" s="91"/>
+      <c r="AO41" s="114"/>
       <c r="AP41" s="16">
         <v>46171</v>
       </c>
       <c r="AQ41" s="29"/>
       <c r="AR41" s="27"/>
-      <c r="AS41" s="94"/>
+      <c r="AS41" s="122"/>
       <c r="AT41" s="16">
         <v>46020</v>
       </c>
       <c r="AU41" s="29"/>
       <c r="AV41" s="29"/>
     </row>
-    <row r="42" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="91"/>
+    <row r="42" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="114"/>
       <c r="B42" s="72">
         <v>45930</v>
       </c>
@@ -4955,7 +4961,7 @@
       <c r="D42" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E42" s="91"/>
+      <c r="E42" s="114"/>
       <c r="F42" s="16">
         <v>46052</v>
       </c>
@@ -4977,7 +4983,7 @@
       <c r="P42" s="24">
         <v>7</v>
       </c>
-      <c r="Q42" s="94"/>
+      <c r="Q42" s="122"/>
       <c r="R42" s="16">
         <v>45960</v>
       </c>
@@ -4985,51 +4991,51 @@
       <c r="T42" s="24">
         <v>7</v>
       </c>
-      <c r="U42" s="91"/>
+      <c r="U42" s="114"/>
       <c r="V42" s="14">
         <v>45899</v>
       </c>
       <c r="W42" s="15"/>
       <c r="X42" s="20"/>
-      <c r="Y42" s="91"/>
+      <c r="Y42" s="114"/>
       <c r="Z42" s="16">
         <v>45930</v>
       </c>
       <c r="AA42" s="23"/>
       <c r="AB42" s="19"/>
-      <c r="AC42" s="94"/>
+      <c r="AC42" s="122"/>
       <c r="AD42" s="16">
         <v>45960</v>
       </c>
       <c r="AE42" s="29"/>
       <c r="AF42" s="27"/>
-      <c r="AG42" s="94"/>
+      <c r="AG42" s="122"/>
       <c r="AH42" s="16">
         <v>45930</v>
       </c>
       <c r="AI42" s="23"/>
       <c r="AJ42" s="27"/>
-      <c r="AK42" s="94"/>
+      <c r="AK42" s="122"/>
       <c r="AL42" s="16">
         <v>46142</v>
       </c>
       <c r="AM42" s="23"/>
       <c r="AN42" s="19"/>
-      <c r="AO42" s="91"/>
+      <c r="AO42" s="114"/>
       <c r="AP42" s="14">
         <v>46172</v>
       </c>
       <c r="AQ42" s="21"/>
       <c r="AR42" s="20"/>
-      <c r="AS42" s="94"/>
+      <c r="AS42" s="122"/>
       <c r="AT42" s="16">
         <v>46021</v>
       </c>
       <c r="AU42" s="29"/>
       <c r="AV42" s="29"/>
     </row>
-    <row r="43" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" s="92"/>
+    <row r="43" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="115"/>
       <c r="B43" s="72" t="s">
         <v>63</v>
       </c>
@@ -5039,7 +5045,7 @@
       <c r="D43" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="E43" s="92"/>
+      <c r="E43" s="115"/>
       <c r="F43" s="14">
         <v>46053</v>
       </c>
@@ -5057,21 +5063,21 @@
       <c r="P43" s="24">
         <v>7</v>
       </c>
-      <c r="Q43" s="94"/>
+      <c r="Q43" s="122"/>
       <c r="R43" s="16"/>
       <c r="S43" s="23"/>
       <c r="T43" s="19"/>
-      <c r="U43" s="92"/>
+      <c r="U43" s="115"/>
       <c r="V43" s="14">
         <v>45900</v>
       </c>
       <c r="W43" s="20"/>
       <c r="X43" s="15"/>
-      <c r="Y43" s="92"/>
+      <c r="Y43" s="115"/>
       <c r="Z43" s="16"/>
       <c r="AA43" s="23"/>
       <c r="AB43" s="19"/>
-      <c r="AC43" s="94"/>
+      <c r="AC43" s="122"/>
       <c r="AD43" s="16">
         <v>45961</v>
       </c>
@@ -5081,24 +5087,24 @@
       <c r="AH43" s="16"/>
       <c r="AI43" s="23"/>
       <c r="AJ43" s="27"/>
-      <c r="AK43" s="94"/>
+      <c r="AK43" s="122"/>
       <c r="AL43" s="16"/>
       <c r="AM43" s="23"/>
       <c r="AN43" s="19"/>
-      <c r="AO43" s="92"/>
+      <c r="AO43" s="115"/>
       <c r="AP43" s="14">
         <v>46173</v>
       </c>
       <c r="AQ43" s="21"/>
       <c r="AR43" s="20"/>
-      <c r="AS43" s="94"/>
+      <c r="AS43" s="122"/>
       <c r="AT43" s="16">
         <v>46022</v>
       </c>
       <c r="AU43" s="29"/>
       <c r="AV43" s="34"/>
     </row>
-    <row r="44" spans="1:48" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:48" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="35"/>
       <c r="B44" s="36"/>
       <c r="C44" s="12" t="s">
@@ -5196,7 +5202,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:48" ht="15" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A45" s="42"/>
       <c r="B45" s="43"/>
       <c r="C45" s="44">
@@ -5315,11 +5321,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B46" s="11"/>
     </row>
-    <row r="47" spans="1:48" x14ac:dyDescent="0.45">
-      <c r="A47" s="109"/>
+    <row r="47" spans="1:48" x14ac:dyDescent="0.25">
+      <c r="A47" s="94"/>
       <c r="B47" s="50"/>
       <c r="C47" s="50"/>
       <c r="D47" s="50"/>
@@ -5368,8 +5374,8 @@
       <c r="AU47" s="51"/>
       <c r="AV47" s="51"/>
     </row>
-    <row r="48" spans="1:48" x14ac:dyDescent="0.45">
-      <c r="A48" s="109"/>
+    <row r="48" spans="1:48" x14ac:dyDescent="0.25">
+      <c r="A48" s="94"/>
       <c r="B48" s="52" t="s">
         <v>40</v>
       </c>
@@ -5420,8 +5426,8 @@
       <c r="AU48" s="51"/>
       <c r="AV48" s="51"/>
     </row>
-    <row r="49" spans="1:48" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A49" s="109"/>
+    <row r="49" spans="1:48" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A49" s="94"/>
       <c r="B49" s="52"/>
       <c r="C49" s="51"/>
       <c r="D49" s="51"/>
@@ -5478,8 +5484,8 @@
       <c r="AU49" s="51"/>
       <c r="AV49" s="51"/>
     </row>
-    <row r="50" spans="1:48" ht="21.4" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A50" s="109"/>
+    <row r="50" spans="1:48" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A50" s="94"/>
       <c r="B50" s="53"/>
       <c r="C50" s="51" t="s">
         <v>41</v>
@@ -5490,22 +5496,22 @@
       <c r="G50" s="51"/>
       <c r="H50" s="51"/>
       <c r="I50" s="51"/>
-      <c r="J50" s="112" t="s">
+      <c r="J50" s="97" t="s">
         <v>42</v>
       </c>
-      <c r="K50" s="113"/>
-      <c r="L50" s="113"/>
-      <c r="M50" s="113"/>
-      <c r="N50" s="113"/>
-      <c r="O50" s="113"/>
-      <c r="P50" s="113"/>
-      <c r="Q50" s="113"/>
-      <c r="R50" s="114"/>
+      <c r="K50" s="98"/>
+      <c r="L50" s="98"/>
+      <c r="M50" s="98"/>
+      <c r="N50" s="98"/>
+      <c r="O50" s="98"/>
+      <c r="P50" s="98"/>
+      <c r="Q50" s="98"/>
+      <c r="R50" s="99"/>
       <c r="S50" s="76"/>
       <c r="T50" s="67" t="s">
         <v>56</v>
       </c>
-      <c r="U50" s="51" t="s">
+      <c r="U50" s="123" t="s">
         <v>84</v>
       </c>
       <c r="V50" s="76"/>
@@ -5540,8 +5546,8 @@
       <c r="AU50" s="51"/>
       <c r="AV50" s="51"/>
     </row>
-    <row r="51" spans="1:48" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A51" s="109"/>
+    <row r="51" spans="1:48" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="94"/>
       <c r="B51" s="54"/>
       <c r="C51" s="51" t="s">
         <v>43</v>
@@ -5552,17 +5558,17 @@
       <c r="G51" s="51"/>
       <c r="H51" s="51"/>
       <c r="I51" s="51"/>
-      <c r="J51" s="115" t="s">
+      <c r="J51" s="100" t="s">
         <v>54</v>
       </c>
-      <c r="K51" s="116"/>
-      <c r="L51" s="116"/>
-      <c r="M51" s="116"/>
-      <c r="N51" s="116"/>
-      <c r="O51" s="116"/>
-      <c r="P51" s="116"/>
-      <c r="Q51" s="116"/>
-      <c r="R51" s="117"/>
+      <c r="K51" s="101"/>
+      <c r="L51" s="101"/>
+      <c r="M51" s="101"/>
+      <c r="N51" s="101"/>
+      <c r="O51" s="101"/>
+      <c r="P51" s="101"/>
+      <c r="Q51" s="101"/>
+      <c r="R51" s="102"/>
       <c r="S51" s="51"/>
       <c r="T51" s="68" t="s">
         <v>19</v>
@@ -5598,29 +5604,29 @@
       <c r="AU51" s="51"/>
       <c r="AV51" s="51"/>
     </row>
-    <row r="52" spans="1:48" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A52" s="109"/>
+    <row r="52" spans="1:48" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A52" s="94"/>
       <c r="B52" s="55"/>
-      <c r="C52" s="110" t="s">
+      <c r="C52" s="95" t="s">
         <v>44</v>
       </c>
-      <c r="D52" s="111"/>
-      <c r="E52" s="111"/>
-      <c r="F52" s="111"/>
-      <c r="G52" s="111"/>
-      <c r="H52" s="111"/>
-      <c r="I52" s="111"/>
-      <c r="J52" s="118" t="s">
+      <c r="D52" s="96"/>
+      <c r="E52" s="96"/>
+      <c r="F52" s="96"/>
+      <c r="G52" s="96"/>
+      <c r="H52" s="96"/>
+      <c r="I52" s="96"/>
+      <c r="J52" s="103" t="s">
         <v>55</v>
       </c>
-      <c r="K52" s="119"/>
-      <c r="L52" s="119"/>
-      <c r="M52" s="119"/>
-      <c r="N52" s="119"/>
-      <c r="O52" s="119"/>
-      <c r="P52" s="119"/>
-      <c r="Q52" s="119"/>
-      <c r="R52" s="120"/>
+      <c r="K52" s="104"/>
+      <c r="L52" s="104"/>
+      <c r="M52" s="104"/>
+      <c r="N52" s="104"/>
+      <c r="O52" s="104"/>
+      <c r="P52" s="104"/>
+      <c r="Q52" s="104"/>
+      <c r="R52" s="105"/>
       <c r="S52" s="77"/>
       <c r="T52" s="69" t="s">
         <v>47</v>
@@ -5656,27 +5662,27 @@
       <c r="AU52" s="51"/>
       <c r="AV52" s="51"/>
     </row>
-    <row r="53" spans="1:48" ht="21" x14ac:dyDescent="0.65">
-      <c r="A53" s="109"/>
+    <row r="53" spans="1:48" ht="21" x14ac:dyDescent="0.35">
+      <c r="A53" s="94"/>
       <c r="B53" s="57"/>
-      <c r="C53" s="110" t="s">
+      <c r="C53" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="D53" s="111"/>
-      <c r="E53" s="111"/>
-      <c r="F53" s="111"/>
-      <c r="G53" s="111"/>
-      <c r="H53" s="111"/>
-      <c r="I53" s="111"/>
-      <c r="J53" s="121"/>
-      <c r="K53" s="121"/>
-      <c r="L53" s="121"/>
-      <c r="M53" s="121"/>
-      <c r="N53" s="121"/>
-      <c r="O53" s="121"/>
-      <c r="P53" s="121"/>
-      <c r="Q53" s="121"/>
-      <c r="R53" s="121"/>
+      <c r="D53" s="96"/>
+      <c r="E53" s="96"/>
+      <c r="F53" s="96"/>
+      <c r="G53" s="96"/>
+      <c r="H53" s="96"/>
+      <c r="I53" s="96"/>
+      <c r="J53" s="106"/>
+      <c r="K53" s="106"/>
+      <c r="L53" s="106"/>
+      <c r="M53" s="106"/>
+      <c r="N53" s="106"/>
+      <c r="O53" s="106"/>
+      <c r="P53" s="106"/>
+      <c r="Q53" s="106"/>
+      <c r="R53" s="106"/>
       <c r="S53" s="77"/>
       <c r="T53" s="70" t="s">
         <v>48</v>
@@ -5712,8 +5718,8 @@
       <c r="AU53" s="51"/>
       <c r="AV53" s="51"/>
     </row>
-    <row r="54" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A54" s="109"/>
+    <row r="54" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="94"/>
       <c r="B54" s="58"/>
       <c r="C54" s="51"/>
       <c r="D54" s="51"/>
@@ -5735,7 +5741,7 @@
       <c r="T54" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="U54" s="51" t="s">
+      <c r="U54" s="123" t="s">
         <v>84</v>
       </c>
       <c r="V54" s="51"/>
@@ -5766,8 +5772,8 @@
       <c r="AU54" s="51"/>
       <c r="AV54" s="51"/>
     </row>
-    <row r="55" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A55" s="109"/>
+    <row r="55" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="94"/>
       <c r="B55" s="58"/>
       <c r="C55" s="51"/>
       <c r="D55" s="51"/>
@@ -5816,64 +5822,64 @@
       <c r="AU55" s="51"/>
       <c r="AV55" s="51"/>
     </row>
-    <row r="56" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="11"/>
     </row>
-    <row r="57" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="11"/>
       <c r="O57" s="47"/>
     </row>
-    <row r="58" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="11"/>
       <c r="O58" s="47"/>
     </row>
-    <row r="59" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="11"/>
       <c r="O59" s="47"/>
     </row>
-    <row r="64" spans="1:48" ht="21" x14ac:dyDescent="0.65">
-      <c r="J64" s="107"/>
-      <c r="K64" s="107"/>
-      <c r="L64" s="107"/>
-      <c r="M64" s="107"/>
-      <c r="N64" s="107"/>
-      <c r="O64" s="107"/>
-      <c r="P64" s="107"/>
-      <c r="Q64" s="107"/>
-      <c r="R64" s="107"/>
-      <c r="S64" s="107"/>
-      <c r="T64" s="107"/>
-      <c r="U64" s="107"/>
+    <row r="64" spans="1:48" ht="21" x14ac:dyDescent="0.35">
+      <c r="J64" s="92"/>
+      <c r="K64" s="92"/>
+      <c r="L64" s="92"/>
+      <c r="M64" s="92"/>
+      <c r="N64" s="92"/>
+      <c r="O64" s="92"/>
+      <c r="P64" s="92"/>
+      <c r="Q64" s="92"/>
+      <c r="R64" s="92"/>
+      <c r="S64" s="92"/>
+      <c r="T64" s="92"/>
+      <c r="U64" s="92"/>
     </row>
-    <row r="66" spans="10:21" ht="21" x14ac:dyDescent="0.65">
-      <c r="J66" s="108"/>
-      <c r="K66" s="108"/>
-      <c r="L66" s="108"/>
-      <c r="M66" s="108"/>
-      <c r="N66" s="108"/>
-      <c r="O66" s="108"/>
-      <c r="P66" s="108"/>
-      <c r="Q66" s="108"/>
-      <c r="R66" s="108"/>
-      <c r="S66" s="108"/>
-      <c r="T66" s="108"/>
-      <c r="U66" s="108"/>
+    <row r="66" spans="10:21" ht="21" x14ac:dyDescent="0.35">
+      <c r="J66" s="93"/>
+      <c r="K66" s="93"/>
+      <c r="L66" s="93"/>
+      <c r="M66" s="93"/>
+      <c r="N66" s="93"/>
+      <c r="O66" s="93"/>
+      <c r="P66" s="93"/>
+      <c r="Q66" s="93"/>
+      <c r="R66" s="93"/>
+      <c r="S66" s="93"/>
+      <c r="T66" s="93"/>
+      <c r="U66" s="93"/>
     </row>
-    <row r="67" spans="10:21" ht="21" x14ac:dyDescent="0.65">
-      <c r="J67" s="108"/>
-      <c r="K67" s="108"/>
-      <c r="L67" s="108"/>
-      <c r="M67" s="108"/>
-      <c r="N67" s="108"/>
-      <c r="O67" s="108"/>
-      <c r="P67" s="108"/>
-      <c r="Q67" s="108"/>
-      <c r="R67" s="108"/>
-      <c r="S67" s="108"/>
-      <c r="T67" s="108"/>
-      <c r="U67" s="108"/>
+    <row r="67" spans="10:21" ht="21" x14ac:dyDescent="0.35">
+      <c r="J67" s="93"/>
+      <c r="K67" s="93"/>
+      <c r="L67" s="93"/>
+      <c r="M67" s="93"/>
+      <c r="N67" s="93"/>
+      <c r="O67" s="93"/>
+      <c r="P67" s="93"/>
+      <c r="Q67" s="93"/>
+      <c r="R67" s="93"/>
+      <c r="S67" s="93"/>
+      <c r="T67" s="93"/>
+      <c r="U67" s="93"/>
     </row>
-    <row r="68" spans="10:21" ht="21" x14ac:dyDescent="0.65">
+    <row r="68" spans="10:21" ht="21" x14ac:dyDescent="0.35">
       <c r="J68" s="56"/>
       <c r="K68" s="56"/>
       <c r="L68" s="56"/>
@@ -5884,16 +5890,80 @@
     </row>
   </sheetData>
   <mergeCells count="100">
-    <mergeCell ref="J64:U64"/>
-    <mergeCell ref="J66:U66"/>
-    <mergeCell ref="J67:U67"/>
-    <mergeCell ref="A47:A55"/>
-    <mergeCell ref="C52:I52"/>
-    <mergeCell ref="C53:I53"/>
-    <mergeCell ref="J50:R50"/>
-    <mergeCell ref="J51:R51"/>
-    <mergeCell ref="J52:R52"/>
-    <mergeCell ref="J53:R53"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="Y34:Y40"/>
+    <mergeCell ref="Y41:Y43"/>
+    <mergeCell ref="E17:E23"/>
+    <mergeCell ref="E24:E30"/>
+    <mergeCell ref="E31:E37"/>
+    <mergeCell ref="E38:E43"/>
+    <mergeCell ref="I14:I20"/>
+    <mergeCell ref="I21:I27"/>
+    <mergeCell ref="I28:I34"/>
+    <mergeCell ref="I35:I40"/>
+    <mergeCell ref="M14:M20"/>
+    <mergeCell ref="M21:M27"/>
+    <mergeCell ref="M28:M34"/>
+    <mergeCell ref="M35:M41"/>
+    <mergeCell ref="Q13:Q17"/>
+    <mergeCell ref="A13:A19"/>
+    <mergeCell ref="A20:A26"/>
+    <mergeCell ref="A27:A33"/>
+    <mergeCell ref="E13:E16"/>
+    <mergeCell ref="AS13:AS19"/>
+    <mergeCell ref="AS20:AS26"/>
+    <mergeCell ref="AS27:AS33"/>
+    <mergeCell ref="AG20:AG26"/>
+    <mergeCell ref="AG27:AG33"/>
+    <mergeCell ref="U13:U15"/>
+    <mergeCell ref="U16:U22"/>
+    <mergeCell ref="U23:U29"/>
+    <mergeCell ref="U30:U36"/>
+    <mergeCell ref="Q25:Q31"/>
+    <mergeCell ref="Q32:Q38"/>
+    <mergeCell ref="A34:A40"/>
+    <mergeCell ref="AS34:AS40"/>
+    <mergeCell ref="AS41:AS43"/>
+    <mergeCell ref="AK13:AK17"/>
+    <mergeCell ref="AK18:AK24"/>
+    <mergeCell ref="AK25:AK31"/>
+    <mergeCell ref="AK32:AK38"/>
+    <mergeCell ref="AK39:AK43"/>
+    <mergeCell ref="AO13:AO15"/>
+    <mergeCell ref="AO16:AO22"/>
+    <mergeCell ref="AO23:AO29"/>
+    <mergeCell ref="AO30:AO36"/>
+    <mergeCell ref="AO37:AO43"/>
+    <mergeCell ref="B9:J9"/>
+    <mergeCell ref="AG13:AG19"/>
+    <mergeCell ref="AK12:AL12"/>
+    <mergeCell ref="AG34:AG40"/>
+    <mergeCell ref="AG41:AG42"/>
+    <mergeCell ref="AC13:AC15"/>
+    <mergeCell ref="AC16:AC22"/>
+    <mergeCell ref="AC23:AC29"/>
+    <mergeCell ref="AC30:AC36"/>
+    <mergeCell ref="AC37:AC43"/>
+    <mergeCell ref="Q39:Q43"/>
+    <mergeCell ref="Q18:Q24"/>
+    <mergeCell ref="AK11:AN11"/>
+    <mergeCell ref="B1:AN1"/>
+    <mergeCell ref="H2:J3"/>
+    <mergeCell ref="S3:AE3"/>
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="B8:J8"/>
+    <mergeCell ref="P8:S8"/>
+    <mergeCell ref="W8:Z8"/>
+    <mergeCell ref="U11:X11"/>
+    <mergeCell ref="Y11:AB11"/>
+    <mergeCell ref="AC11:AF11"/>
+    <mergeCell ref="AG11:AJ11"/>
+    <mergeCell ref="AO12:AP12"/>
+    <mergeCell ref="U37:U43"/>
+    <mergeCell ref="Y13:Y19"/>
+    <mergeCell ref="Y20:Y26"/>
+    <mergeCell ref="Y27:Y33"/>
+    <mergeCell ref="AG12:AH12"/>
     <mergeCell ref="AS12:AT12"/>
     <mergeCell ref="Q11:T11"/>
     <mergeCell ref="A11:D11"/>
@@ -5910,80 +5980,16 @@
     <mergeCell ref="Y12:Z12"/>
     <mergeCell ref="AC12:AD12"/>
     <mergeCell ref="AO11:AR11"/>
-    <mergeCell ref="U37:U43"/>
-    <mergeCell ref="Y13:Y19"/>
-    <mergeCell ref="Y20:Y26"/>
-    <mergeCell ref="Y27:Y33"/>
-    <mergeCell ref="AG12:AH12"/>
-    <mergeCell ref="U11:X11"/>
-    <mergeCell ref="Y11:AB11"/>
-    <mergeCell ref="AC11:AF11"/>
-    <mergeCell ref="AG11:AJ11"/>
-    <mergeCell ref="AO12:AP12"/>
-    <mergeCell ref="B1:AN1"/>
-    <mergeCell ref="H2:J3"/>
-    <mergeCell ref="S3:AE3"/>
-    <mergeCell ref="B7:J7"/>
-    <mergeCell ref="B8:J8"/>
-    <mergeCell ref="P8:S8"/>
-    <mergeCell ref="W8:Z8"/>
-    <mergeCell ref="B9:J9"/>
-    <mergeCell ref="AG13:AG19"/>
-    <mergeCell ref="AK12:AL12"/>
-    <mergeCell ref="AG34:AG40"/>
-    <mergeCell ref="AG41:AG42"/>
-    <mergeCell ref="AC13:AC15"/>
-    <mergeCell ref="AC16:AC22"/>
-    <mergeCell ref="AC23:AC29"/>
-    <mergeCell ref="AC30:AC36"/>
-    <mergeCell ref="AC37:AC43"/>
-    <mergeCell ref="Q39:Q43"/>
-    <mergeCell ref="Q18:Q24"/>
-    <mergeCell ref="AK11:AN11"/>
-    <mergeCell ref="AS34:AS40"/>
-    <mergeCell ref="AS41:AS43"/>
-    <mergeCell ref="AK13:AK17"/>
-    <mergeCell ref="AK18:AK24"/>
-    <mergeCell ref="AK25:AK31"/>
-    <mergeCell ref="AK32:AK38"/>
-    <mergeCell ref="AK39:AK43"/>
-    <mergeCell ref="AO13:AO15"/>
-    <mergeCell ref="AO16:AO22"/>
-    <mergeCell ref="AO23:AO29"/>
-    <mergeCell ref="AO30:AO36"/>
-    <mergeCell ref="AO37:AO43"/>
-    <mergeCell ref="A13:A19"/>
-    <mergeCell ref="A20:A26"/>
-    <mergeCell ref="A27:A33"/>
-    <mergeCell ref="E13:E16"/>
-    <mergeCell ref="AS13:AS19"/>
-    <mergeCell ref="AS20:AS26"/>
-    <mergeCell ref="AS27:AS33"/>
-    <mergeCell ref="AG20:AG26"/>
-    <mergeCell ref="AG27:AG33"/>
-    <mergeCell ref="U13:U15"/>
-    <mergeCell ref="U16:U22"/>
-    <mergeCell ref="U23:U29"/>
-    <mergeCell ref="U30:U36"/>
-    <mergeCell ref="Q25:Q31"/>
-    <mergeCell ref="Q32:Q38"/>
-    <mergeCell ref="A34:A40"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="Y34:Y40"/>
-    <mergeCell ref="Y41:Y43"/>
-    <mergeCell ref="E17:E23"/>
-    <mergeCell ref="E24:E30"/>
-    <mergeCell ref="E31:E37"/>
-    <mergeCell ref="E38:E43"/>
-    <mergeCell ref="I14:I20"/>
-    <mergeCell ref="I21:I27"/>
-    <mergeCell ref="I28:I34"/>
-    <mergeCell ref="I35:I40"/>
-    <mergeCell ref="M14:M20"/>
-    <mergeCell ref="M21:M27"/>
-    <mergeCell ref="M28:M34"/>
-    <mergeCell ref="M35:M41"/>
-    <mergeCell ref="Q13:Q17"/>
+    <mergeCell ref="J64:U64"/>
+    <mergeCell ref="J66:U66"/>
+    <mergeCell ref="J67:U67"/>
+    <mergeCell ref="A47:A55"/>
+    <mergeCell ref="C52:I52"/>
+    <mergeCell ref="C53:I53"/>
+    <mergeCell ref="J50:R50"/>
+    <mergeCell ref="J51:R51"/>
+    <mergeCell ref="J52:R52"/>
+    <mergeCell ref="J53:R53"/>
   </mergeCells>
   <phoneticPr fontId="19" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -5994,6 +6000,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100862694ECED4E1948B5E8D6F6BADC8D0D" ma:contentTypeVersion="4" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="504949a71aab2cb719442a6beb0a4eda">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="102bceca-7b01-449b-a089-7caeaaf28d79" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="029f89eff23996dad8873f8cabf28cb6" ns2:_="">
     <xsd:import namespace="102bceca-7b01-449b-a089-7caeaaf28d79"/>
@@ -6137,22 +6158,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81A92264-ACEF-4D40-97BD-271C523DAB22}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="102bceca-7b01-449b-a089-7caeaaf28d79"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14055206-B539-47B6-8443-C51626AAA311}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8BE1D94A-FAA5-446A-9E63-96728E017CDA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6168,28 +6198,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14055206-B539-47B6-8443-C51626AAA311}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81A92264-ACEF-4D40-97BD-271C523DAB22}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="102bceca-7b01-449b-a089-7caeaaf28d79"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>